<commit_message>
feat: ejecutable nativo para macOS ProcesStudio.app e incorporacion de historia de usuario PST-022
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -976,9 +976,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>PST-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Packaging &amp; Compatibilidad macOS</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Lanzador Nativo Portable para macOS (ProcesStudio.app)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Como usuario del sistema operativo Apple macOS (Macbook / iMac), quiero disponer de un paquete de aplicación nativo ProcesStudio.app ejecutable con doble clic y totalmente funcional, para abrir mis proyectos de procesos JSON en macOS con la misma facilidad que en Windows.</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Creación del bundle oficial ProcesStudio.app con estructura estándar Contents/Info.plist y Contents/MacOS/ProcesStudio.
+2. Ejecutable nativo compatible con procesadores Intel y Apple Silicon (M1/M2/M3/M4).
+3. Resolución automática de la carpeta ../Proyectos/ para persistencia local de archivos .json.
+4. Soporte complementario del script ProcesStudio_Mac.command para ejecución por terminal.</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: renderizado de impresion multipagina centrado para Flujograma en PDF y registro de historia PST-023
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1002,9 +1002,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>PST-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Flujograma &amp; Impresión</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Renderizador de Impresión Multipágina Vectorial para Flujograma en PDF</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Como usuario administrativo, quiero que al imprimir el diagrama de flujo en PDF la salida esté perfectamente centrada, oculte la interfaz de la aplicación y se extienda a lo largo de tantas páginas A4 como sea necesario con saltos limpios sin cortar tarjetas, para obtener un documento impreso profesional y completo.</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Ocultamiento total de la barra de navegación Header durante la impresión mediante clase print:hidden.
+2. Motor de renderizado vectorial FlowchartPrintDocument con estructura descendente nivel por nivel.
+3. Centrado automático horizontal de cada nivel en la hoja A4 con flechas SVG continuas y etiquetas de condición.
+4. Soporte nativo de paginación vertical con reglas page-break-inside: avoid en cada bloque.
+5. Selector de Vista Paginada para previsualizar el PDF en pantalla antes de imprimir.</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: sistema de historial Deshacer y Rehacer paso a paso e historia PST-024
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1029,9 +1029,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>PST-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Edición &amp; Productividad</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Sistema de Historial Deshacer (Ctrl+Z) y Rehacer (Ctrl+Y) Paso a Paso</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Como usuario y modelador de procesos, quiero poder deshacer y rehacer con Ctrl+Z y Ctrl+Y (o mediante botones en la barra superior) cada uno de los movimientos y modificaciones realizadas en la sesión paso a paso, para rectificar errores o experimentar con el diagrama con total libertad y seguridad.</v>
+      </c>
+      <c r="E25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Registro inmutable de instantáneas previas (snapshots) en una pila de historial con límite de hasta 50 estados.
+2. Captura única de estado al iniciar arrastre de tarjetas (onNodeDragStart) evitando saturación de memoria.
+3. Deshacer (Ctrl+Z) y Rehacer (Ctrl+Y / Ctrl+Shift+Z) paso a paso en movimientos, adición/eliminación de nodos, conexiones, cambios de estilo y carriles.
+4. Botones visuales Deshacer y Rehacer en la barra superior (Header) con estados activos/deshabilitados e información contextual.
+5. Aislamiento de eventos de teclado en inputs y textareas para preservar el deshacer nativo de texto.</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: paginacion vertical y saltos de hoja irrestrictos en PDF de flujograma e historia PST-025
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1056,9 +1056,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>PST-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Flujograma &amp; Impresión</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Paginación Vertical y Saltos de Hoja Irrestrictos en PDF de Flujograma</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Como usuario y auditor de calidad, quiero que al imprimir el Flujograma en PDF la salida se expanda de forma natural y automática a lo largo de tantas páginas A4 como demande la extensión del diagrama, para que ningún nivel o actividad sea truncado a una sola hoja por restricciones de altura o desborde del lienzo.</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Reseteo global de altura, posicionamiento y overflow en @media print para todos los ancestros SPA (html, body, #root, .h-screen, main, .overflow-*).
+2. Estructuración en bloques naturales independientes (.flowchart-level-block) con break-inside: avoid y page-break-inside: avoid.
+3. Contenedor de impresión dedicado (.flowchart-print-container) con ancho al 100% y visualización limpia sin solapamientos.
+4. Soporte de exportación a PDF multipágina probado y verificado tanto en navegadores como en Electron portable.</v>
+      </c>
+      <c r="F26" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: suite de 6 modulos avanzados offline e historias PST-026 a PST-031
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G32"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1082,9 +1082,165 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>PST-026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Calidad ISO 9001 &amp; Auditoría BPMN</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Auditor de Calidad y Linter Topológico BPMN 2.0 / ISO 9001 con Score de Salud</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Como auditor de calidad y oficial de cumplimiento, quiero una herramienta de diagnóstico en 1-clic que escanee todo el diagrama BPMN 2.0 y evalúe la completitud normativa (eventos iniciales/finales, compuertas sin salida, actividades sin rol o SLA, ciclos infinitos y controles de riesgo), asignando un puntaje de salud del 0 al 100% y permitiendo saltar directamente a la tarjeta infractora, para garantizar procesos 100% conformes y sin errores estructurales.</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Motor linter determinista offline que analiza nodos, conexiones, SLAs, riesgos y roles sin requerir internet.
+2. Cálculo de puntuación de salud (Health Score 0-100%) con clasificación visual (Excelente, Bueno, Regular, Crítico).
+3. Clasificación de hallazgos por severidad (Crítico / Error, Advertencia, Sugerencia).
+4. Botón "Localizar" en cada hallazgo que centra y resalta automáticamente la tarjeta en el lienzo.</v>
+      </c>
+      <c r="F27" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>PST-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Lienzo &amp; Colaboración</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Notas Adhesivas (Sticky Notes / Post-its) en el Lienzo</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Como analista o facilitador de talleres de procesos, quiero agregar notas adhesivas flotantes (post-its) de colores con texto libre en cualquier área de la pizarra, para registrar comentarios de reuniones, dudas operativas o recordatorios de diseño sin alterar la lógica formal del flujo BPMN.</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Nuevo elemento interactivo "Nota Adhesiva" arrastrable desde la paleta lateral.
+2. Edición de texto inline instantánea al hacer foco o doble clic en la nota.
+3. Selector dinámico de colores de fondo estilo post-it (amarillo, azul, verde, rosa, púrpura, naranja).
+4. Exclusión transparente del flujo de secuencia BPMN formal pero guardado persistente en el archivo JSON del proyecto.</v>
+      </c>
+      <c r="F28" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>PST-028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Gobernanza Organizacional</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Matriz RACI Interactiva y Exportación a Excel (.xlsx)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Como gerente o líder de transformación, quiero una pestaña con la Matriz RACI (Responsable, Aprobador, Consultado, Informado) calculada automáticamente cruzando actividades y roles, con edición de celdas en tiempo real y exportación directa a Excel (.xlsx), para clarificar el gobierno de responsabilidades del proceso.</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pestaña independiente "Matriz RACI" en la barra de navegación principal.
+2. Cálculo matricial automático cruzando cada actividad con los roles operativos del proceso.
+3. Interactividad para alternar asignaciones (R, A, C, I o vacío) con clic en celda.
+4. Exportación directa a hoja de cálculo Excel (.xlsx) 100% offline con formato corporativo y leyendas claras.</v>
+      </c>
+      <c r="F29" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>PST-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Interoperabilidad &amp; Exportación</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Centro Unificado de Exportación Multiformato (PNG 300 DPI, SVG, BPMN 2.0 XML, Word .doc)</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Como profesional de procesos, quiero un centro de exportación centralizado que me permita descargar mi proyecto en imágenes de alta resolución (PNG 300 DPI / SVG vectorial), archivo estándar XML BPMN 2.0 (ISO 19510) y manual operativo en Microsoft Word (.doc), para compartir mi trabajo con cualquier herramienta corporativa sin depender de conexión a internet.</v>
+      </c>
+      <c r="E30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Modal unificado "Centro de Exportación" accesible desde el menú superior.
+2. Exportación a imagen PNG HD y SVG vectorial escalable sin pérdida de nitidez.
+3. Generación de archivo BPMN 2.0 XML estándar (ISO 19510) compatible con Camunda, Signavio y Bizagi.
+4. Generación y descarga de Manual de Procedimientos en formato Microsoft Word (.doc) con tablas e índice formal.</v>
+      </c>
+      <c r="F30" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>PST-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Simulación &amp; Optimización</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Simulador de Procesos con Detección de Cuellos de Botella y Mapa de Calor (Heatmap)</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Como ingeniero de optimización o Black Belt Lean, quiero ejecutar simulaciones de eventos discretos con diferentes volúmenes de casos y turnos de trabajo para identificar cuellos de botella y colorear un mapa de calor dinámico sobre el lienzo, para saber dónde se concentran las colas de espera y tiempos muertos.</v>
+      </c>
+      <c r="E31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Simulador de eventos discretos con parámetros configurables (número de casos, horas diarias, capacidad de recursos).
+2. Detección automática de la actividad que representa el cuello de botella crítico y cálculo de costos y tiempos de espera.
+3. Botón "Aplicar Mapa de Calor en el Lienzo" que tiñe los nodos de verde (rápido) a rojo intenso (saturado/crítico).
+4. Botón de 1-clic para restaurar los colores originales del proyecto.</v>
+      </c>
+      <c r="F31" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>PST-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Control de Versiones &amp; Auditoría</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Comparador Visual de Versiones JSON (Visual Diff Tool)</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Como auditor o líder de proyecto, quiero comparar el proyecto actual con cualquier versión previa o archivo JSON externo para ver un resumen de actividades agregadas, modificadas o eliminadas y diferencias campo por campo, para auditar cambios antes de publicar una nueva versión.</v>
+      </c>
+      <c r="E32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Modal de comparación con selector de archivo JSON de versión previa o base.
+2. Análisis comparativo instantáneo mostrando métricas de elementos añadidos, eliminados y modificados.
+3. Tabla detallada con etiquetas de colores (verde para agregados, rojo para eliminados, ámbar para modificados).
+4. Inspección expandible campo por campo destacando valor anterior vs. valor actual.</v>
+      </c>
+      <c r="F32" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(diagram): agregar hojas de impresion multi-pagina y exportacion a pdf (PST-032)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1238,9 +1238,37 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>PST-032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Diseño &amp; Exportación de Diagramas</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Sistema de Hojas de Impresión Multi-Página (Recuadros Punteados A4/Carta/A3) y Exportación PDF</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Como analista o líder de procesos, quiero configurar recuadros punteados en el lienzo que delimiten hojas de impresión en formatos estándar (A4, Carta, A3 en horizontal/vertical) pudiendo moverlos y ajustarlos a gusto, para generar un documento PDF de alta calidad que contenga todas las hojas configuradas con nomenclatura estandarizada sin hojas en blanco.</v>
+      </c>
+      <c r="E33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Recuadros punteados interactivos en el lienzo con identificación de hoja (Hoja 1, Hoja 2, etc.), arrastre para reposicionar y tiradores en esquinas para redimensionar.
+2. Selector de formatos de hoja (A4, Carta, A3) y orientaciones (Horizontal / Vertical).
+3. Botones de acción rápida: "+ Agregar Hoja", "Auto-Encuadrar" y "Ocultar Hojas".
+4. Generación nativa en cliente de PDF multi-página mediante jsPDF sin hojas en blanco ni distorsiones.
+5. Nomenclatura automática de archivo PDF con referencia al proyecto: AAAA-MM-DD_proc-&lt;codigo&gt;_&lt;titulo&gt;_diagrama.pdf.
+6. Integración en el Centro de Exportación y en el visor de Diagrama del Proceso.</v>
+      </c>
+      <c r="F33" t="str">
+        <v>2026-09-17</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G32"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(routing): enrutamiento inteligente con evasion automatica de obstaculos y bucles (PST-033)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1266,9 +1266,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>PST-033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Lienzo BPMN &amp; Enrutamiento</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Enrutamiento Inteligente con Evasión Automática de Obstáculos en Conexiones BPMN</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Como modelador y documentador de procesos, quiero que las líneas de conexión (Sequence Flow) esquiven automáticamente cualquier tarjeta o nodo intermedio sin pasar nunca por encima ni por debajo de ellos, adaptándose en tiempo real durante el arrastre y diseño del lienzo, para mantener flujos visualmente impecables, legibles y 100% profesionales.</v>
+      </c>
+      <c r="E34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Motor de enrutamiento ortogonal A* integrado que detecta cajas delimitadoras de tarjetas con margen de seguridad de 22px.
+2. Evasión reactiva y suave en tiempo real al arrastrar, crear o desplazar nodos y compuertas.
+3. Esquinas con redondeo ergonómico (fillets de 10px) y trayectorias sin cruces invasivos sobre elementos.
+4. Soporte unificado en lienzo interactivo y vista de impresión/exportación multi-página a PDF.
+5. Exclusión inteligente de contenedores de carril (PoolLanes) para permitir que los flujos transiten libremente por el fondo de los carriles.</v>
+      </c>
+      <c r="F34" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(presentation): seccion de modo presentacion dinamica prezi con zoom y panel ordenado (PST-034)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1293,9 +1293,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>PST-034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Presentación &amp; Navegación</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Modo Presentación Dinámica e Interactiva tipo Prezi con Zoom Animado y Panel de Contenido Ordenado</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Como expositor, auditor o analista de procesos, quiero una sección de presentación inmersiva que recorra el diagrama paso a paso con animaciones de cámara cinemáticas (zoom dinámico centrado en cada tarjeta) y un panel lateral derecho estructurado con todo el contenido del paso (responsable, SLA, sistemas TI, entradas/salidas, riesgos y normativa), para exponer y capacitar sobre los flujos de trabajo de forma clara, ordenada y profesional.</v>
+      </c>
+      <c r="E35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Extractor de secuencia topológica automática que ordena las actividades desde el Evento de Inicio hasta el Fin respetando bifurcaciones y carriles.
+2. Animación fluida de cámara (ReactFlow setCenter con zoom 1.35) y resplandor focal (spotlight) sobre la tarjeta activa con atenuación del entorno.
+3. Panel lateral derecho estructurado con código estándar, rol, título, descripción, métricas de tiempo/SLA, sistemas TI, entradas (inputs), entregables (outputs), marco legal/ISO 9001, riesgos operativos y enlaces de navegación del flujo.
+4. Barra de reproducción flotante con controles de Inicio, Anterior, Siguiente, selector de diapositivas y modo Auto-Play con temporizador configurable.
+5. Control completo por teclado (←, →, Espacio para pausar/reanudar, Home, End, F para pantalla completa, Esc para salir y F5/Shift+P para abrir desde el lienzo).</v>
+      </c>
+      <c r="F35" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G35"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(header): barra superior compacta con menus desplegables e iconos profesionales (PST-035)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1320,9 +1320,37 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>PST-035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Navegación &amp; Experiencia de Usuario</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Reestructuración y Compactación de Barra Superior con Menús Desplegables Profesionales</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Como usuario de ProcesStudio en pantallas estándar o portátiles, quiero una barra superior limpia y compacta organizada en menús desplegables jerárquicos (Vistas &amp; Matrices, Herramientas) y botones de utilidad en iconos con tooltip, para acceder a todas las 18 funcionalidades del sistema con 1 solo clic sin desborde horizontal ni necesidad de múltiples monitores.</v>
+      </c>
+      <c r="E36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Pestañas de acceso directo para "Proyectos" y "Lienzo BPMN".
+2. Menú desplegable flotante "Vistas &amp; Matrices" que agrupa Flujograma, Matriz SIPOC, Matriz RACI y Documento &amp; Reporte.
+3. Menú desplegable flotante "Herramientas" que agrupa Presentación Prezi (F5), Auditor de Calidad, Simulador de Flujos, Comparador de Versiones y Navegador de Subprocesos.
+4. Grupo de utilidades compactas en formato icono con tooltip (Deshacer, Rehacer, Ver Carpeta, Temas y Modo Claro/Oscuro).
+5. Acciones principales destacadas (Exportar, Nuevo y Guardar con indicador animado de cambios pendientes).
+6. Reducción de más del 65% del ancho total de la barra con cierre automático al hacer clic afuera (click outside listener).</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): botones icon-only, separacion contenido/estilo y correccion de presentacion (PST-036)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1348,9 +1348,34 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>PST-036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>UI / UX &amp; Presentación</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Iconos Compactos en Encabezado, Separación de Propiedades (Contenido vs Estilo) y Visibilidad de Elementos en Presentación</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Como modelador de procesos, quiero botones de acción icon-only en la barra superior, un panel lateral derecho organizado con pestañas dedicadas para Contenido/Datos y Estilo/Apariencia, y una visualización destacada y en primer plano de todos los elementos durante el modo presentación tipo Prezi, para tener una experiencia de diseño ágil, limpia y sin interferencias visuales.</v>
+      </c>
+      <c r="E37" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Los botones de Exportar, Nuevo y Guardar en la cabecera superior muestran exclusivamente sus iconos representativos con tooltips contextuales y estados de guardado/animación.
+2. El panel lateral de propiedades de nodos separa limpiamente la edición de información BPMN (ID, Título, Descripción, Rol, SLA, SIPOC, Riesgos) y personalización visual (Paletas de color, opacidad, bordes, encabezados, tipografía, orientación y bloqueo de dimensiones) mediante pestañas "Contenido &amp; Datos" y "Estilo &amp; Apariencia".
+3. Corrección de la jerarquía de capas (z-index y ordenamiento de nodos de fondo a primer plano: Swimlane -&gt; Subproceso -&gt; Tareas -&gt; Compuertas -&gt; Eventos) en el modo presentación tipo Prezi para garantizar que todas las tarjetas de proceso sean visibles con nitidez y resplandor activo sobre los carriles.</v>
+      </c>
+      <c r="F37" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(sync): sistema de versionado multi-equipo y carga automatica de ultima version (PST-037)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1373,9 +1373,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>PST-037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Sincronización &amp; Versionado Multi-Equipo</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Sistema de Versionado Inmutable Multi-Equipo (Casa/Trabajo), Agrupación de Macroprocesos y Detección Automática de Última Versión</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Como usuario que modela procesos alternando entre la PC de su casa y la del trabajo mediante sincronización con Git, quiero que la aplicación guarde las nuevas versiones o revisiones como archivos inmutables independientes y agrupe automáticamente los procesos en el Gestor permitiéndome abrir con un solo clic la versión más reciente disponible, para erradicar por completo los conflictos de merge en Git y trabajar de forma transparente y segura entre múltiples dispositivos.</v>
+      </c>
+      <c r="E38" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Creación del servicio processVersionManager para cálculo de semver, normalización de claves canónicas y agrupación inteligente de archivos JSON en ProcessGroupSummary.
+2. La tarjeta de proyecto en el Dashboard agrupa todas las versiones de un mismo proceso, destacando un badge "vX.X (Última versión)", botón primario "Abrir Última Versión" y acordeón desplegable con el historial completo de archivos y revisiones.
+3. Incorporación del modal NewRevisionModal en el encabezado para guardar nuevas versiones inmutables con incremento semántico (Menor, Parche, Mayor), etiqueta de dispositivo (PC Casa, PC Trabajo, Personalizado) y descripción de cambios para trazabilidad ISO 9001.
+4. Integración del banner NewerVersionBanner en el lienzo BPMN que detecta si el archivo cargado tiene una versión más nueva sincronizada en disco y ofrece actualizarla al instante con un clic.</v>
+      </c>
+      <c r="F38" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(presentation): selector de color de fondo y trama en modo presentacion (PST-038)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1399,9 +1399,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>PST-038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>UI / UX &amp; Presentación</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Personalización de Color de Fondo, Trasparencia y Trama de Cuadrícula en Modo Presentación (Prezi)</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Como presentador o expositor de procesos ante autoridades, quiero personalizar el color de fondo del lienzo en modo presentación (eligiendo entre presets como Negro Profundo OLED, Grafito Slate, Blanco Puro, Gris Papel, o un color HEX personalizado) y alternar el tipo de cuadrícula (puntos, líneas, cruces o liso), para adaptar la estética visual a proyectores, salas de reuniones o pantallas OLED con máxima legibilidad.</v>
+      </c>
+      <c r="E39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Incorporación de menú desplegable con botón de paleta en la cabecera del Modo Presentación con 6 presets optimizados (OLED, Slate, Midnight, Blanco Puro, Gris Papel, Crema Cálido) y selector nativo de color HEX.
+2. Selector de trama de fondo dinámico que permite alternar entre variantes Dots, Lines, Cross y None (liso).
+3. Cálculo automático de contraste para el color de los puntos/líneas de la cuadrícula según la luminancia del fondo.
+4. Persistencia automática de la configuración de fondo en localStorage para conservar las preferencias del expositor en sesiones futuras.</v>
+      </c>
+      <c r="F39" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(presentation): orden secuencial manual y tiempos individuales por paso (PST-039)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1425,9 +1425,37 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>PST-039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Presentación &amp; Navegación</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Orden Secuencial Manual y Tiempos Individuales por Paso en Modo Presentación</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Como expositor y facilitador de procesos, quiero poder definir un número de orden secuencial manual en las actividades (manteniendo el orden topológico automático por defecto) y fijar una duración específica en segundos para cada paso durante el modo Auto-Play, para adaptar el ritmo y la narrativa de la presentación a pasos complejos o introductorios sin quedar limitado a un único temporizador global.</v>
+      </c>
+      <c r="E40" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Propiedades de nodo presentationOrder (número de orden secuencial) y presentationDurationSeconds (duración en segundos) en BpmnNodeData.
+2. Extractor de secuencia topológica que prioriza los números de orden manuales cuando están definidos y utiliza el orden de flujo y geometría por defecto cuando no lo están.
+3. Panel de Propiedades del Nodo en la pestaña "Contenido &amp; Datos" con sección dedicada "Modo Presentación (Secuencia &amp; Tiempo)".
+4. Panel lateral del Modo Presentación con control directo en vivo para ajustar el número de orden y tiempo de permanencia del paso activo.
+5. Temporizador dinámico de Auto-Play que sincroniza automáticamente el tiempo restante con la duración individual de cada tarjeta o el tiempo base global seleccionado.
+6. Línea de tiempo con scrubber dots diferenciados para pasos con duración individual e indicador de tiempo restante vs tiempo total del paso.</v>
+      </c>
+      <c r="F40" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(git): ignorar y desindexar archivos de proyectos locales (PST-040)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1453,9 +1453,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>PST-040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Gestión de Versiones y Repositorio / Proyectos</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Exclusión de Archivos de Proyectos Locales de Git (.gitignore)</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Como usuario y desarrollador de ProcesStudio, quiero que Git ignore y desindexe los archivos JSON de proyectos de procesos en la carpeta de proyectos, para evitar que el trabajo y modificaciones locales de proyectos generen cambios o conflictos innecesarios en el control de versiones del código fuente.</v>
+      </c>
+      <c r="E41" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Configuración de directivas en .gitignore para ignorar archivos en MiAppProcesos_USB/Proyectos/* y Proyectos/*.
+2. Conservación del directorio en el repositorio mediante el marcador .gitkeep.
+3. Desindexación en Git de los archivos JSON de proyectos previamente rastreados sin borrarlos del disco local (git rm --cached).
+4. Verificación de que crear o editar proyectos JSON no genere avisos en git status.
+5. Preservación física intacta de los archivos existentes en la máquina local.</v>
+      </c>
+      <c r="F41" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): navegacion por clic en minimapa, formas BPMN fieles y etiqueta marco (PST-041)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1480,9 +1480,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>PST-041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Lienzo BPMN &amp; Minimapa / UI</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Navegación Interactiva por Clic en Minimapa, Representación Geométrica BPMN Fiel y Ajuste de Etiqueta Marco</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Como modelador de procesos, quiero navegar por el lienzo haciendo clic o arrastrando directamente en el minimapa, ver la silueta geométrica real de cada elemento (círculos para eventos, rombos para compuertas y rectángulos para tareas) e identificar el marco legal como "Marco" en las propiedades de la tarjeta, para tener una orientación espacial precisa y una interfaz limpia.</v>
+      </c>
+      <c r="E42" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Clic en cualquier área del minimapa desplaza y centra suavemente la vista del lienzo hacia esas coordenadas (setCenter con animación).
+2. Clic directo sobre un nodo en el minimapa centra la vista en dicho nodo y lo selecciona automáticamente abriendo su panel de propiedades.
+3. Soporte para arrastre (pannable) y zoom con la rueda del ratón (zoomable) directo en el minimapa.
+4. Eventos de inicio, fin, checkpoint de calidad y temporizador se representan con silueta circular concéntrica en el minimapa.
+5. Compuertas exclusivas y paralelas se representan fielmente como rombos/diamantes.
+6. Nodos seleccionados muestran contorno activo y resplandor de alta visibilidad.
+7. La etiqueta "Marco Legal" en el panel lateral de propiedades se actualiza a "Marco".</v>
+      </c>
+      <c r="F42" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G42"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): insercion centrada, subprocesos multinivel N niveles y estandares BPMN (PST-042)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1509,9 +1509,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>PST-042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Lienzo BPMN &amp; Subprocesos Multinivel</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Inserción en Centro de Pantalla, Subprocesos Multinivel Recursivos (N Niveles) y Estandarización Gráfica BPMN</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Como modelador y arquitecto de procesos, quiero que los nuevos elementos añadidos desde la paleta aparezcan en el centro del viewport visible actual, poder ingresar recursivamente a cualquier subproceso para ver y editar su diagrama interno con su distribución original (permitiendo anidar subprocesos hasta N niveles de profundidad con navegación adelante/atrás fluida), y que todas las figuras sigan rigurosamente las normas estándar de diagramación de procesos BPMN 2.0 / ISO 5807 (marcador [+] de subproceso colapsado, eventos circulares y compuertas en rombo), para diseñar arquitecturas de procesos jerárquicas complejas con máxima ergonomía y rigor normativo.</v>
+      </c>
+      <c r="E43" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Los nuevos elementos creados desde la barra lateral se ubican dinámicamente en el centro exacto de la pantalla/viewport actual del usuario considerando el nivel de zoom y desplazamiento (pan) mediante screenToFlowPosition.
+2. Ingreso a subprocesos con doble clic sobre la tarjeta, mediante el botón estándar BPMN [+] en la base o mediante la acción explícita "Ingresar" en el pie de la tarjeta.
+3. Soporte multinivel recursivo para anidar subprocesos dentro de otros subprocesos hasta N niveles de profundidad sin restricciones de arquitectura.
+4. Al ingresar a un subproceso comprimido previamente, se restauran las tarjetas en su distribución y coordenadas relativas espaciales originales.
+5. Barra de navegación jerárquica (Breadcrumbs) superior fija en el lienzo que muestra la ruta completa de niveles (Inicio &gt; Subproceso A &gt; Subproceso B...), botón de retorno rápido al nivel anterior y salto directo a cualquier nivel intermedio.
+6. Plena capacidad de edición en cualquier nivel interno del subproceso: agregar actividades, conectar flechas, editar propiedades, crear nuevos subprocesos internos y eliminar elementos.
+7. Cumplimiento de estándares de modelado BPMN 2.0: marcador oficial [+] en base de subprocesos colapsados, eventos de inicio en círculo simple, eventos de fin en círculo grueso y compuertas en rombo.</v>
+      </c>
+      <c r="F43" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(subprocess): aislamiento contextual de subprocesos anidados y paneles en nivel activo (PST-043)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1538,9 +1538,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>PST-043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Subprocesos &amp; Jerarquías Recursivas</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Aislamiento Contextual de Creación, Compresión y Edición en Subprocesos Anidados (N Niveles)</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Como modelador de procesos, quiero que al crear, comprimir, descomprimir o editar subprocesos y elementos estando dentro de un subproceso, los cambios se apliquen estricta y exclusivamente en el lienzo del subproceso activo actual en vez de volcarse sobre el proceso principal raíz, para garantizar la consistencia jerárquica de diagramas anidados complejos.</v>
+      </c>
+      <c r="E44" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. La acción de comprimir actividades seleccionadas en un subproceso (compressSelection) opera sobre el grafo del nivel activo (getActiveGraph) reemplazando los nodos únicamente dentro del subproceso actual mediante updateGraphForPath.
+2. La descompresión de subprocesos (decompressSubProcess) despliega las actividades directamente en el nivel donde se encuentra ubicado el nodo.
+3. La creación de nuevos subprocesos (addNode) pre-inicializa de inmediato su estructura interna subProcessCanvas y subProcessSteps con flujo estándar inicial persistido.
+4. El panel lateral de propiedades (PropertiesPanel) lee y edita los nodos y conectores del grafo activo sin importar el nivel de profundidad del subproceso.
+5. La barra de herramientas de selección (SelectionToolbar), las acciones de copiar/pegar y el modal de compresión respetan el contexto del subproceso activo.</v>
+      </c>
+      <c r="F44" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G44"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(lanes): personalizacion completa y gestion dinamica de carriles organizativos (PST-044)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1565,9 +1565,37 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>PST-044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Carriles Organizativos &amp; Swimlanes</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Personalización Integral y Gestión Dinámica de Carriles Organizativos (Swimlanes)</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Como modelador y analista de procesos, quiero personalizar libremente las opciones de carriles organizativos (swimlanes), pudiendo crear nuevos carriles, editar nombres de áreas, roles responsables, sistemas TI y colores tanto desde el panel de propiedades como desde un modal centralizado de gestión, para reflejar fielmente la estructura departamental y organizativa de la institución.</v>
+      </c>
+      <c r="E45" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. El selector de Carril Organizativo (Swimlane) en el panel de propiedades incluye acciones rápidas para crear nuevo carril (+ Nuevo), editar el carril activo (Editar) y acceder a la administración global (⚙ Gestionar).
+2. El menú desplegable incorpora las opciones interactivas "+ Crear nuevo carril..." y "⚙ Gestionar y reordenar carriles...".
+3. Editor rápido en línea en el panel de propiedades para modificar nombre de área, rol/puesto responsable, sistema informático y color de carril con actualización en tiempo real.
+4. Formulario en línea para crear y asignar un nuevo carril directamente a la actividad seleccionada en un solo paso.
+5. Modal integral de gestión (ManageLanesModal) con listado completo de carriles, reordenamiento vertical (subir/bajar), edición detallada, alta de nuevos carriles con selector de paleta y eliminación segura con reasignación automática de actividades.
+6. Sincronización bidireccional automática: los cambios de carriles impactan en cascada en todas las tarjetas de actividad vinculadas, en los carriles de fondo del lienzo y en las matrices SIPOC y RACI.</v>
+      </c>
+      <c r="F45" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G45"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): generalizacion de interfaz, herramientas, responsable, marco y carriles desde cero (PST-045)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1593,9 +1593,39 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>PST-045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Generalización de Interfaz, Herramientas, Responsable y Carriles desde Cero</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Transición a Herramientas, Nuevo Campo Responsable, Conservación de Marco, Plazos Activables, Carriles por Título y Experiencia Generalizada</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Como usuario y modelador de procesos, quiero una experiencia generalizada libre de menciones forzadas a normas ISO o prescripciones legales, donde las tarjetas nuevas tengan campos limpios con texto de guía sutil en gris ("detrás" del cursor sin tener que borrar ejemplos previos), los proyectos comiencen con 0 carriles para crearlos únicamente por título desde cero con memoria por proceso, los plazos sean opcionales y activables con interruptor, y el concepto "Sistema TI" se denomine "Herramienta", conservando el campo "Marco" para normas o procedimientos aplicables.</v>
+      </c>
+      <c r="E46" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sustitución transversal del término y concepto "Sistema TI" por "Herramienta" (con icono de herramienta Wrench) en paneles de propiedades, tarjetas del lienzo, paleta lateral y modales.
+2. Incorporación del nuevo campo "Responsable" en el modelo de datos, tarjeta del lienzo (con icono User) y panel de propiedades.
+3. Preservación del campo "Marco" (data.legalFramework) para encuadre normativo, procedimental o de instructivos con marcador de posición genérico.
+4. Proyectos nuevos inician con 0 carriles organizativos (lanes: []) con memoria y persistencia por proyecto en formato JSON.
+5. Creación de carriles en un solo paso solicitando únicamente el Título del carril (con paleta de color opcional) en PropertiesPanel, ManageLanesModal y SwimlaneBackground.
+6. Plazo de ejecución activable/desactivable mediante casilla interactiva con etiquetas generalizadas ("Plazo de Ejecución", "Plazo Estricto / Crítico") ocultando insignias SLA cuando está inactivo.
+7. Eliminación de todas las referencias normativas rígidas (ISO 9001, ISO 8601, ISO 19510, prescripción legal) en textos visibles de la interfaz.
+8. Textos predeterminados limpios en tarjetas y formularios: campos inicializados en vacío con texto en gris (placeholder) sin ejemplos ("ej:") permitiendo escribir inmediatamente sin necesidad de borrar.</v>
+      </c>
+      <c r="F46" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G46"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: campo Link en tarjetas, nomenclatura jerarquica Pxx-Nxx y barra permanente de procesos anidados
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1623,9 +1623,40 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
+        <v>PST-046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Jerarquías de Proceso</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Campo Link en Tarjetas, Nomenclatura Jerárquica Pxx-Nxx y Barra Permanente de Procesos Anidados</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Como usuario y analista de procesos, quiero que las tarjetas posean un campo Link con botón directo para abrir enlaces web o documentación externa en el navegador, que las Service Tasks se diferencien de las User Tasks (SRV vs TSK), que todas las tarjetas utilicen una nomenclatura jerárquica con código de proceso y nivel (P01-N00-..., P02-N01-...), y que la barra superior de navegación entre procesos anidados permanezca disponible en todo momento con siglas compactas (P01N00, P02N01) que se expanden al seleccionarlas mostrando título y nivel.</v>
+      </c>
+      <c r="E47" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Nuevo campo Link en el modelo BpmnNodeData, editable en PropertiesPanel con icono, campo URL y botón de prueba rápida.
+2. Pequeño botón interactivo con icono ExternalLink en la cabecera de las tarjetas (TaskNode y SubProcessNode) que abre la URL en el navegador externo predeterminado sin seleccionar ni mover la tarjeta.
+3. Nomenclatura específica y diferenciada para tareas de servicio (SRV) frente a tareas de usuario (TSK).
+4. Nomenclaturas estructuradas por código de proceso y nivel de anidamiento: P01-N00-TSK-01 para el proceso padre, y numeración secuencial única para cada nuevo subproceso (P02-N01-TSK-01, P02-N01-SRV-01, etc.).
+5. Pre-inicialización de flujos estándar de nuevos subprocesos con la nomenclatura jerárquica correspondiente a su código y nivel.
+6. Barra de navegación superior fija y permanente en el lienzo que nunca desaparece al estar en el proceso padre.
+7. Los procesos no seleccionados se muestran con sus siglas compactas (P01N00, P02N01, P03N01...) y navegan directamente al hacer clic.
+8. El proceso seleccionado actualmente se expande mostrando su icono distintivo (Home/Layers), sigla, título y nivel (Nivel 0, Nivel 1...).
+9. Botón Volver para subir un nivel cuando se encuentra dentro de un subproceso anidado.</v>
+      </c>
+      <c r="F47" t="str">
+        <v>2026-10-15</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: punto de control interactivo de contracurva y curvatura en conexiones (PST-047)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1654,9 +1654,39 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
+        <v>PST-047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Enrutamiento de Conexiones</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Punto de Control Interactivo de Contracurva en Conexiones con Snapping Magnético</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Como modelador y diagramador de procesos, quiero un punto de control interactivo en el centro de las líneas de conexión que me permita manipular el lugar exacto donde realiza la contracurva (quiebre o transición vertical) tanto en el eje X como arquearla en el eje Y, para poder alinear visualmente múltiples caídas verticales que convergen en una misma tarjeta y esquivar obstáculos o tarjetas intermedias con curvas Bézier armónicas.</v>
+      </c>
+      <c r="E48" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Punto de control circular interactivo en el centro de las líneas de flujo (SequenceFlowEdge) visible al seleccionar la línea o pasar el cursor por encima.
+2. Arrastre bidireccional libre (X, Y) con cursor interactivo grab/grabbing y retroalimentación táctil/visual en tiempo real.
+3. Desplazamiento horizontal (eje X) que modula el lugar exacto de la contracurva (punto de inflexión) permitiendo alinear perfectamente las caídas verticales de múltiples líneas que ingresan a un mismo nodo.
+4. Desplazamiento vertical (eje Y) que genera un arco bicúbico C1 suave para rodear o esquivar tarjetas intermedias sin quiebres ni esquinas agudas.
+5. Snapping magnético automático en el eje X: se atrae a los puntos de contracurva de líneas vecinas a menos de 10px para facilitar una alineación visual perfecta.
+6. Restablecimiento instantáneo de curvatura automática mediante doble clic sobre el punto de control o mediante el botón "Restablecer" en el panel de propiedades.
+7. Soporte completo de historial Deshacer / Rehacer (Ctrl+Z / Ctrl+Y) antes de cada manipulación.
+8. Persistencia garantizada en el esquema JSON del proyecto (edge.data.controlPoint: { x, y }) y reflejo idéntico en las exportaciones gráficas SVG/PNG.</v>
+      </c>
+      <c r="F48" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="G48" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): rodeo automatico de tarjetas y ajuste de hasta 4 puntos en conexiones (PST-048)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1684,9 +1684,39 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
+        <v>PST-048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Enrutamiento de Conexiones</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Rodeo Automático de Tarjetas y Ajuste Multi-Punto (1 a 4) en Conexiones</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Como modelador y diagramador de procesos, quiero que las conexiones que se dirigen hacia atrás rodeen automáticamente las tarjetas sin atravesarlas, y poder definir entre 1 y 4 puntos de control en las propiedades de la conexión para manipular libremente la trayectoria de la línea en el lienzo.</v>
+      </c>
+      <c r="E49" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Rodeo automático perimetral: cuando una tarjeta se conecta hacia otra que está antes en el flujo (conexión retrógrada o bucle de retorno), la conexión rodea el exterior de las tarjetas origen, destino e intermedias por encima o por debajo con margen de seguridad sin atravesar ningún nodo.
+2. Selector de cantidad de puntos en PropertiesPanel: permite configurar 1, 2, 3 o 4 puntos de ajuste (por defecto 1 punto) con persistencia en el proyecto.
+3. Manejadores interactivos multi-punto en el lienzo (SequenceFlowEdge): se muestran de 1 a 4 puntos identificados numéricamente (1..4) al seleccionar o pasar el cursor sobre la línea.
+4. Arrastre independiente y suave: cada punto se puede desplazar en X e Y de forma independiente con cálculo de curvatura continua C1 (spline bicúbico/multicúbico Bézier).
+5. Snapping magnético por punto: alineación automática con puntos de control de conexiones vecinas a menos de 10px.
+6. Restablecimiento flexible: doble clic en el lienzo o botón "Restablecer" en el panel de propiedades para volver al trazado automático perimetral.
+7. Fidelidad idéntica en exportaciones: el motor de generación SVG (imageExportService) replica exactamente la trayectoria perimetral y los puntos de control configurados.
+8. Integración con Deshacer/Rehacer (Ctrl+Z / Ctrl+Y) y esquema de persistencia JSON en proyectos.</v>
+      </c>
+      <c r="F49" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(standards): estandarizacion de denominadores de 3 letras para todos los nodos (PST-049)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1714,9 +1714,41 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
+        <v>PST-049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Estandarización BPMN &amp; Denominadores de 3 Letras</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Estandarización Universal de Denominadores de 3 Letras para Todos los Nodos BPMN</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Como arquitecto y modelador de procesos, quiero que cada tipo de evento, tarjeta, compuerta o ítem del proceso cuente siempre con su propio denominador estándar unívoco de exactamente 3 letras, diferenciando explícitamente eventos de inicio (INI) y fin (FIN), compuertas exclusivas (GTW) y paralelas (PAR), puntos de control de calidad (QCP), carriles (CAR) y notas adhesivas (NOT), para asegurar una nomenclatura jerárquica homogénea, predecible y sin colisiones en los códigos de identificación de todo el sistema.</v>
+      </c>
+      <c r="E50" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Diferenciación estricta de eventos: StartEvent asigna prefijo INI (ej. P01-N00-INI-01) y EndEvent asigna FIN (ej. P01-N00-FIN-01).
+2. Diferenciación de compuertas: ExclusiveGateway utiliza GTW y ParallelGateway utiliza PAR.
+3. Puntos de control de calidad estandarizados a 3 letras: QualityCheckpointEvent utiliza QCP (ej. P01-N00-QCP-01).
+4. Carriles organizacionales (Swimlanes) estandarizados a 3 letras: PoolLane utiliza CAR (ej. P01-N00-CAR-01).
+5. Notas adhesivas / Post-its estandarizadas a 3 letras: StickyNote utiliza NOT (ej. P01-N00-NOT-01).
+6. Coherencia con tareas preexistentes de 3 letras: UserTask (TSK), ServiceTask (SRV), ManualTask (MNL), TimerBoundaryEvent (TMR) y SubProcess (SUB).
+7. Generación automática y correlativa en processHierarchyService.formatHierarchicalStandardId() respetando los nuevos denominadores.
+8. Actualización de plantillas de nuevos subprocesos en useCanvasStore y proyectos predeterminados en defaultProjects.
+9. Actualización de insignias de fallback en todos los componentes visuales de nodo (StartEventNode, EndEventNode, GatewayNode, QualityCheckpointNode, SwimlaneNode, StickyNoteNode y TaskNode).
+10. Actualización de filtros de calidad en el navegador jerárquico de procesos (ProcessHierarchyNavigator).</v>
+      </c>
+      <c r="F50" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): posicionamiento deslizable de etiquetas sobre linea de conexion (PST-050)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1746,9 +1746,39 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
+        <v>PST-050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Enrutamiento de Conexiones</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Posicionamiento Deslizable y Ajuste Interactivo de Etiquetas sobre la Línea de Conexión</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Como modelador y diagramador de procesos, quiero poder modificar la posición de la etiqueta de cualquier conexión arrastrándola directamente en el lienzo o mediante un deslizador en el panel de propiedades, asegurando que permanezca siempre situada sobre la línea de conexión adaptándose a su curvatura o al movimiento de las tarjetas conectadas.</v>
+      </c>
+      <c r="E51" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Arrastre directo en el lienzo: la etiqueta de conexión (conditionText) cuenta con cursor interactivo grab/grabbing e icono sutil GripVertical, permitiendo arrastrarla a lo largo de la línea.
+2. Restricción estricta sobre la trayectoria: el algoritmo getClosestRatioOnSvgPath proyecta la posición del cursor directamente sobre el trazo SVG de la conexión, asegurando que la pastilla de la etiqueta se mantenga 100% sobre la línea en todo momento.
+3. Propiedad paramétrica relativa: se almacena la posición como proporción (labelPosition entre 0.05 y 0.95), garantizando que si se mueven las tarjetas o se modifica la curvatura de la línea, la etiqueta mantenga su posición relativa sobre el trazo.
+4. Control en PropertiesPanel: deslizador porcentual de posición (5% a 95%), botones de salto rápido (Inicio 20%, Centro 50%, Final 80%) y botón Centrar para restablecer la etiqueta al punto medio.
+5. Restablecimiento rápido: doble clic sobre la etiqueta en el lienzo para devolverla al centro de la línea.
+6. Integración con Deshacer/Rehacer (Ctrl+Z / Ctrl+Y) antes de cada manipulación.
+7. Fidelidad idéntica en exportaciones gráficas SVG, PNG y PDF (imageExportService y pdfDiagramExportService).
+8. Persistencia garantizada en el esquema JSON de proyectos.</v>
+      </c>
+      <c r="F51" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): notas redimensionables con vinculo a tarjeta y resaltado jerarquico (PST-051)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1776,9 +1776,40 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
+        <v>PST-051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Jerarquía de Procesos</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Resaltado Progresivo en Barra de Procesos, Notas Redimensionables y Vinculación con Tarjeta</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Como analista y modelador de procesos, quiero que la barra de navegación de procesos resalte en un color degradado con opacidad progresiva la ruta de anidación donde estoy parado (opacándose más hacia la raíz), y en las notas adhesivas poder redimensionar su tamaño libremente, vincularlas opcionalmente a cualquier tarjeta del diagrama mediante una línea punteada y que el campo Responsable se complete automáticamente con el asignado a dicha tarjeta vinculada, para contar con una clara orientación contextual jerárquica y una documentación contextual ágil y articulada con las actividades.</v>
+      </c>
+      <c r="E52" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Barra de navegación jerárquica (SubProcessBreadcrumbs): cálculo de distancia jerárquica de cada elemento de la ruta activa respecto al nivel actual.
+2. Resaltado cromático progresivo: el proceso actual en el que se está parado se destaca con el color de acento y fondo al 100%, mientras que los procesos contenedores/ancestros reducen proporcionalmente su opacidad hasta la raíz, dejando las ramas paralelas en tono neutral.
+3. Notas adhesivas redimensionables (StickyNoteNode): integración de NodeResizer con límites mínimos (160x110px), permitiendo ajustar libremente ancho y alto en el lienzo.
+4. Vinculación opcional con tarjeta: selector desplegable en PropertiesPanel para asociar una nota a cualquier tarjeta o ítem del proceso activo, o conexión directa entre conectores en el lienzo.
+5. Conector punteado de asociación: línea de transición discontinua (strokeDasharray: "4,4") sin punta de flecha ni obligatoriedad de asignación.
+6. Herencia automática de Responsable: el pie de la nota refleja en tiempo real el Responsable de la tarjeta asociada (o su rol funcional) y se actualiza ante cualquier modificación.
+7. Si la nota no está vinculada, permite ingresar o mostrar un responsable manual o el texto "Sin responsable".
+8. Exportación gráfica fiel: soporte de dimensiones redimensionadas y líneas punteadas de asociación en exportaciones SVG, PNG y PDF (imageExportService y pdfDiagramExportService).
+9. Persistencia de campos en el archivo de proyecto JSON (relatedNodeId y isAssociation).</v>
+      </c>
+      <c r="F52" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G52"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(canvas): correccion de loop en tarjetas cercanas y movimiento suave de nodos (PST-052)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1807,9 +1807,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53" t="str">
+        <v>PST-052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Enrutamiento de Conexiones</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Corrección de Bucle en Conexiones Cercanas y Movimiento Suave de Nodos</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Como diseñador y modelador de procesos, quiero que las conexiones entre tarjetas que se encuentran muy cerca no formen bucles o rodeos inferiores indeseados, y que el movimiento de las tarjetas al arrastrarlas sea completamente fluido, suave y sin encasillarse de forma trabada, quedando exactamente colocadas en las coordenadas donde las suelto, para diagramar con máxima precisión visual y comodidad de uso.</v>
+      </c>
+      <c r="E53" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enrutamiento en tarjetas cercanas: las conexiones horizontales estándar (Right -&gt; Left) con targetX &gt; sourceX se procesan siempre como flujo directo hacia adelante sin importar la proximidad entre tarjetas.
+2. Supresión de falsos bucles retrógrados: isBackwardConnection solo se activa cuando la tarjeta destino está efectivamente situada detrás de la de origen (targetX &lt;= sourceX).
+3. Cálculo proporcional de curvatura: los puntos de control Bezier escalan con la distancia efectiva (Math.max(4, Math.min(distance * 0.45, 140))), evitando sobrepasos o nudos cuando las tarjetas están pegadas.
+4. Movimiento fluido 60 FPS: eliminación de la atracción magnética invasiva que forzaba a las tarjetas de actividad a saltar bruscamente entre ranuras predefinidas durante el arrastre.
+5. Posicionamiento milimétrico exacto: las tarjetas quedan colocadas exactamente donde el usuario suelta el cursor del ratón.
+6. Supresión de latencia CSS: eliminación de transition-all en contenedores de nodos y desactivación de transiciones espaciales en .react-flow__node, logrando una respuesta 1:1 instantánea.
+7. Preservación del acoplamiento 0px entre carriles (PoolLane) y de las guías visuales punteadas de alineación (AlignmentGuidesOverlay).</v>
+      </c>
+      <c r="F53" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(canvas): eliminar barra flotante superpuesta a navegacion de procesos (PST-053)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1836,9 +1836,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54" t="str">
+        <v>PST-053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Barra de Navegación</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Eliminación de Barra Flotante Superpuesta para Despeje de la Navegación de Procesos</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Como usuario y diagramador de procesos, quiero que al copiar elementos o interactuar con el lienzo no aparezca una barra flotante superpuesta sobre la barra de navegación de procesos (breadcrumbs), para que el hilo jerárquico de procesos se mantenga siempre visible y despejado sin obstrucciones visuales.</v>
+      </c>
+      <c r="E54" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Desmontaje completo de SelectionToolbar: eliminación del componente flotante en ProcessCanvas, suprimiendo la barra persistente que emergía al poblar el portapapeles.
+2. Despeje total de la barra de navegación: los breadcrumbs de subprocesos (SubProcessBreadcrumbs) permanecen 100% visibles y libres de superposición en toda su extensión horizontal.
+3. Preservación integral de atajos de copiar y pegar: las combinaciones universales Ctrl+C y Ctrl+V continúan funcionando fluidamente con notificaciones toast informativas.
+4. Mantenimiento de acciones de control: las funciones de fijado, compresión de subprocesos, orientación y eliminación permanecen plenamente disponibles en el panel de propiedades lateral (PropertiesPanel) y controles superiores.</v>
+      </c>
+      <c r="F54" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G54"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): centrado inteligente y enfoque en start event al entrar a subproceso (PST-054)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1862,9 +1862,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55" t="str">
+        <v>PST-054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Enfoque de Subprocesos</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Centrado Inteligente y Enfoque en Start Event al Entrar a un Subproceso</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Como analista y diagramador de procesos, quiero que siempre que ingrese o navegue a un subproceso la vista del lienzo centre automáticamente el proceso lo más posible, y en caso de que el proceso sea muy largo para el nivel de zoom actual, sitúe automáticamente la primera ficha de evento de inicio (Start Event) al centro vertical y a la izquierda de la pantalla, para visualizar de forma óptima e inmediata la secuencia del flujo de trabajo.</v>
+      </c>
+      <c r="E55" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Detección automática al navegar en subprocesos: el visor ejecuta el centrado inteligente al ingresar a un subproceso o cambiar de nivel jerárquico (subProcessPath.length &gt; 0).
+2. Exclusión de carriles organizacionales: el cálculo del cuadro delimitador del proceso (bounding box) excluye los nodos PoolLane de fondo, considerando únicamente las tarjetas operativas (tareas, compuertas, eventos y notas).
+3. Centrado suave en procesos que caben en pantalla: si el ancho del proceso cabe dentro del ancho visible de la ventana al nivel de zoom actual, la cámara se centra suavemente (setCenter) en el punto medio exacto del proceso sin alterar el zoom.
+4. Enfoque al centro a la izquierda para procesos extensos: si el proceso es más largo que el ancho disponible de la pantalla al zoom actual, la primera ficha Start Event (o el nodo más a la izquierda si no hubiese evento de inicio) se posiciona centrada en el eje Y (viewportHeight / 2) y a la izquierda en el eje X con margen visual cómodo (~140-180px).
+5. Respeto al zoom del usuario: se preserva el nivel de zoom actual del lienzo sin reducciones forzadas ni saltos abruptos.
+6. Estabilidad de edición: el efecto no interfiere ni reposiciona la cámara mientras el usuario arrastra nodos, edita propiedades o modela dentro del subproceso.
+7. Transición animada fluida: la transición de cámara se realiza con una interpolación suave (duration: 400ms).</v>
+      </c>
+      <c r="F55" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G55"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ui): ajuste de alto contraste en textos de la barra de procesos (PST-055)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1891,9 +1891,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="56" xml:space="preserve">
+      <c r="A56" t="str">
+        <v>PST-055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Jerarquía de Procesos</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Ajuste de Colores y Alto Contraste en Textos de la Barra de Navegación de Procesos</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Como analista y modelador de procesos, quiero que los textos de la barra de navegación de subprocesos resalten con nitidez y alto contraste independientemente de si uso un tema claro o un tema oscuro, diferenciando claramente el proceso activo, los procesos ancestros en la ruta jerárquica y los procesos inactivos, para leer e interactuar cómodamente con el árbol de procesos en todo momento.</v>
+      </c>
+      <c r="E56" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Detección automática de luminosidad: el componente SubProcessBreadcrumbs adapta su paleta cromática en tiempo real según el tema activo (isDark de useUiStore).
+2. Máximo contraste en modo claro (Sandpaper, Nordic Studio): los procesos ancestros muestran texto índigo profundo (#312e81) y bordes definidos (#4f46e5), eliminando textos lavanda pálidos casi invisibles.
+3. Resalte premium en proceso activo: sigla en negro azulado (text-indigo-950 font-black), título nítido (text-slate-900) e insignia de nivel en pastilla sólida de alto impacto (bg-indigo-600 text-white font-bold).
+4. Definición en procesos inactivos: texto reforzado en text-slate-700 con efecto hover text-indigo-700.
+5. Visibilidad nocturna en modo oscuro: texto índigo luminoso (#e0e7ff) en ancestros y blanco brillante en proceso activo con bordes de alta visibilidad.
+6. Botón de retorno (Volver): texto contrastado en text-slate-800 (modo claro) y text-slate-100 (modo oscuro) con bordes reforzados.
+7. Separadores chevron: visibilidad mejorada en ambas modalidades cromáticas.</v>
+      </c>
+      <c r="F56" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): propagacion global de estilos en mismo tipo a procesos padre y anidados (PST-056)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1920,9 +1920,39 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="57" xml:space="preserve">
+      <c r="A57" t="str">
+        <v>PST-056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Personalización de Tarjetas</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Propagación Jerárquica Global de Estilos de Tarjeta en "Mismo tipo"</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Como modelador y diseñador de procesos, quiero que al aplicar un cambio de color, tema predefinido o estilo con la opción "Mismo tipo" seleccionada, la modificación se propague a todas las tarjetas del mismo tipo en todo el proyecto, abarcando los procesos padre (nivel raíz y superiores) y los procesos anidados (subprocesos hijos y ramas paralelas), para mantener una identidad visual y taxonomía homogénea en todo el mapa de procesos corporativo.</v>
+      </c>
+      <c r="E57" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Alcance jerárquico universal para Mismo tipo: al seleccionar Mismo tipo (same_type) en el panel de propiedades, las modificaciones cromáticas se propagan por todo el árbol del proyecto (currentProject).
+2. Soporte para procesos padre: las tarjetas del mismo tipo ubicadas en la raíz o en niveles superiores adquieren inmediatamente el nuevo estilo.
+3. Soporte para subprocesos anidados: la función updateNodesDeep recorre recursivamente todos los subprocesos (subProcessCanvas.nodes) e instantáneas comprimidas (compressedSnapshot.nodes) a cualquier nivel N de profundidad.
+4. Propiedades estilísticas contempladas: color de fondo, opacidad, color de borde, color de cabecera, modo de visualización, orientación y dimensiones.
+5. Preservación de carriles: los carriles organizacionales (PoolLane) no se ven alterados ni sobreescritos por la propagación de estilos de tarjetas operativas.
+6. Ámbito individual preservado: la opción "Solo este" continúa afectando de manera exclusiva a la tarjeta seleccionada en el nivel activo.
+7. Soporte para el ámbito "Todos": la opción "Todos" actualiza todas las tarjetas operativas en todo el modelo jerárquico manteniendo homogeneidad global.
+8. Integración con Deshacer/Rehacer (Ctrl+Z / Ctrl+Y): se genera un snapshot de historial atómico para revertir o rehacer la modificación global en un solo paso.</v>
+      </c>
+      <c r="F57" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): centrado inteligente y enfoque en start event en proceso padre y raiz (PST-057)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1950,9 +1950,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="58" xml:space="preserve">
+      <c r="A58" t="str">
+        <v>PST-057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Enfoque de Procesos</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Centrado Inteligente y Enfoque en Start Event para Procesos Padre y Raíz</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Como analista y diagramador de procesos, quiero que el centrado inteligente y enfoque en la primera ficha Start Event se aplique también al proceso principal (raíz) y al regresar a cualquier proceso padre en la jerarquía, asegurando una experiencia de visualización coherente, predecible y orientada al inicio del flujo en todos los niveles del proyecto.</v>
+      </c>
+      <c r="E58" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Cobertura universal de niveles: el efecto de centrado se activa ante cualquier cambio de nivel jerárquico, incluyendo la navegación a subprocesos hijos, el ascenso a procesos padre ("Volver") y el retorno al proceso raíz.
+2. Encuadre al inicio del flujo en procesos extensos: si el proceso padre o raíz es más ancho que la ventana al nivel de zoom actual, la primera ficha Start Event se sitúa centrada verticalmente (viewportHeight / 2) y a la izquierda de la pantalla (~140-180px) para comenzar a leer el diagrama naturalmente hacia la derecha.
+3. Centrado geométrico en diagramas breves: si el proceso padre o raíz cabe dentro de la ventana al nivel de zoom actual, la vista centra la totalidad de las tarjetas operativas de forma suave.
+4. Exclusión de carriles (PoolLane): los swimlanes de fondo no deforman el cálculo de dimensiones ni el posicionamiento del flujo operativo.
+5. Preservación estricta del zoom: el nivel de zoom configurado por el usuario no se modifica ni se resetea.
+6. Estabilidad durante el modelado: el centrado no se re-ejecuta mientras el usuario arrastra tarjetas, crea conexiones o edita propiedades dentro del mismo nivel de proceso.
+7. Carga inicial orientada: al abrir un proyecto, el proceso raíz se encuadra automáticamente de forma óptima sin necesidad de desplazamientos manuales.</v>
+      </c>
+      <c r="F58" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(navigation): boton volver a la izquierda de P01N00 y enfoque en tarjeta de subproceso (PST-058)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -1979,9 +1979,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="59" xml:space="preserve">
+      <c r="A59" t="str">
+        <v>PST-058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Lienzo BPMN 2.0 &amp; Navegación de Subprocesos</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Botón Volver a la Izquierda de P01N00 y Enfoque en Tarjeta de Subproceso Asociada</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Como modelador y analista de procesos, quiero que en la barra de navegación de procesos exista un botón para "Volver" situado inmediatamente a la izquierda del botón de raíz P01N00, y que al hacer clic en él la vista regrese al proceso anterior centrándose exactamente sobre la tarjeta de subproceso asociada y seleccionándola, para retomar el contexto de diagramación de forma ágil, precisa y sin pérdidas de orientación visual.</v>
+      </c>
+      <c r="E59" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Reubicación del botón Volver: el botón se posiciona en el extremo izquierdo de la barra de navegación (SubProcessBreadcrumbs), antes del botón del proceso raíz P01N00.
+2. Estado contextual atenuado: cuando el usuario se encuentra en el proceso principal (raíz), el botón permanece deshabilitado (disabled) con tooltip explicativo para indicar que ya se está en el nivel superior.
+3. Activación al anidar: al ingresar a cualquier subproceso (Nivel 1 o superior), el botón Volver se habilita con contraste elevado y borde interactivo.
+4. Enfoque exacto en la tarjeta de subproceso asociada: al hacer clic en Volver, leaveSubProcess identifica el ID de la tarjeta contenedora en el proceso padre y la cámara se centra suavemente (setCenter, 450ms) en sus coordenadas exactas en lugar de reiniciarse en el Start Event del proceso padre.
+5. Selección y realce visual: la tarjeta de subproceso asociada queda automáticamente seleccionada (selectNode), destacando en el lienzo.
+6. Supresión de duplicidad: se elimina el botón Volver del extremo derecho de la barra de navegación jerárquica.
+7. Soporte para navegación por migas de pan: al hacer clic en un proceso ancestro mediante los breadcrumbs, también se preserva el enfoque en la tarjeta de subproceso correspondiente.</v>
+      </c>
+      <c r="F59" t="str">
+        <v>2026-10-19</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G58"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: habilitar despliegue web universal en GitHub Pages e importacion de proyectos JSON (PST-059)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2008,9 +2008,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="60" xml:space="preserve">
+      <c r="A60" t="str">
+        <v>PST-059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Despliegue Web &amp; Portabilidad Universal</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Despliegue Web Universal en GitHub Pages y Portabilidad Multiplataforma (Zero-Config Municipal)</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Como analista y modelador de procesos, quiero poder abrir ProcesStudio desde la web en cualquier computador (en el trabajo, en mi casa o desde dispositivos móviles) mediante una URL pública con HTTPS y flujo de despliegue automatizado en GitHub Pages, para modelar y auditar procesos sin depender de la red municipal, sin requerir permisos de firewall institucional y pudiendo importar/exportar proyectos JSON con total interoperabilidad.</v>
+      </c>
+      <c r="E60" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Flujo automatizado de CI/CD en GitHub Actions (.github/workflows/deploy.yml) que compila y publica en GitHub Pages tras cada commit en main.
+2. Inmunidad a restricciones de la Red Municipal: no requiere IP pública, ni puertos abiertos en routers institucionales, ni mantener encendida la PC municipal.
+3. Base URL relativa ('./') compatible con ejecución en Electron portable y en la raíz o subdirectorios de GitHub Pages.
+4. Soporte nativo para importar archivos JSON en el Dashboard (botón 'Importar JSON') permitiendo subir flujos creados en cualquier PC o pendrive.
+5. Descarga y exportación ágil de proyectos JSON directamente al computador en la versión Web.
+6. Distintivo contextual dinámico en el Dashboard que indica 'Entorno Web Cloud' o 'Entorno Portable USB' según la plataforma de ejecución.
+7. Persistencia segura y desacoplada en localStorage con compatibilidad total con la estructura de proyectos BPMN 2.0 e ISO 9001:2015.</v>
+      </c>
+      <c r="F60" t="str">
+        <v>2026-10-20</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G60"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: establecer gestion de actas y wisecx como proyectos predeterminados (PST-060)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2037,9 +2037,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="61" xml:space="preserve">
+      <c r="A61" t="str">
+        <v>PST-060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Gestión de Proyectos &amp; Datos Oficiales</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Estandarización de Proyectos Predeterminados Oficiales (Gestión de Actas y WiseCX)</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Como analista de procesos del Tribunal de Faltas y DGSTI, quiero que el sistema incluya por defecto los proyectos oficiales auténticos ("Proceso de Gestión de Actas" y "Procedimiento de Atención, Soporte y Gestión de Incidencias Técnicas - WiseCX") en lugar de datos de prueba genéricos, para que cualquier usuario o colega que acceda a la versión web o portable disponga de inmediato de los flujos de trabajo institucionales reales.</v>
+      </c>
+      <c r="E61" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sustitución de datos demo en defaultProjects.ts por las estructuras JSON oficiales completas de "Gestión de Actas" y "WiseCX".
+2. Depuración automática en el navegador (initializeStorage) de registros obsoletos de proyectos ficticios antiguos.
+3. Inicialización inmediata con los dos procesos reales al abrir la web en cualquier equipo nuevo o al restablecer la memoria local.
+4. Integridad total de metadatos de control documental (autor: Edgar Gonzalez de Prada, códigos PRC-3517 y PRC-DGSTI-2026-001, normativas y swimlanes operativos).
+5. Conservación de los 3 archivos JSON de proyectos oficiales en la carpeta física MiAppProcesos_USB/Proyectos/.</v>
+      </c>
+      <c r="F61" t="str">
+        <v>2026-10-20</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G60"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(database): persistencia cloud en Neon PostgreSQL serverless con sincronizacion local (PST-061)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G62"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2064,9 +2064,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="62" xml:space="preserve">
+      <c r="A62" t="str">
+        <v>PST-061</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Persistencia Cloud &amp; PostgreSQL Serverless</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Persistencia Cloud en PostgreSQL Administrado (Neon Serverless) con Sincronización JSON y Fallback Híbrido</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Como analista de procesos y líder de equipo, quiero que ProcesStudio soporte conexión directa a una base de datos PostgreSQL Serverless (Neon.tech) con compresión JSONB y columnas de métricas indexadas, para consultar el catálogo de procesos en tiempo real (&lt; 2ms) desde cualquier equipo, sincronizar proyectos locales en 1 clic y mantener un respaldo offline híbrido y transparente.</v>
+      </c>
+      <c r="E62" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Integración del cliente oficial @neondatabase/serverless comunicando consultas parametrizadas sobre HTTPS sin requerir backend intermedio.
+2. Arquitectura de datos híbrida: metadatos atómicos e indexados para el Dashboard (título, código, Lead Time, riesgos y QC) y columna graph_data JSONB comprimida con TOAST para el grafo BPMN completo.
+3. Script DDL optimizado (scripts/neon_schema.sql) con extensiones uuid-ossp, pg_trgm, índices GIN y búsqueda léxica tsvector en español.
+4. Persistencia híbrida y dual-write: los proyectos se guardan localmente (USB/localStorage) y se replican automáticamente en Neon si está configurado.
+5. Modal de Base de Datos en el Dashboard con prueba de conectividad y latencia de red en tiempo real.
+6. Sincronizador masivo de 1 clic para migrar proyectos de la unidad USB y del navegador hacia la nube.
+7. Fallback resiliente: ante ausencia de internet o credenciales, la app continúa operativa en modo local sin pérdida de funcionalidad.</v>
+      </c>
+      <c r="F62" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): boton flotante '+' y menu radial circular para conectar proximo nodo (PST-062)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G63"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2093,9 +2093,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="63" xml:space="preserve">
+      <c r="A63" t="str">
+        <v>PST-062</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Modelado Rápido &amp; Experiencia de Canvas (BPMN 2.0)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Botón Quick-Add '+' Flotante y Menú Radial Circular de Próximo Nodo con Conexión Automática</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Como modelador y analista de procesos, quiero que al seleccionar cualquier nodo operativo en el lienzo aparezca un botón '+' a su derecha y que al presionarlo o arrastrarlo se despliegue un menú circular con opciones de nodos BPMN para crear y conectar automáticamente el siguiente elemento del flujo con un solo gesto.</v>
+      </c>
+      <c r="E63" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Botón flotante '+' sincronizado en tiempo real a la derecha del nodo seleccionado mediante NodeToolbar de @xyflow/react.
+2. Exclusión automática de carriles funcionales (PoolLane) y notas adhesivas (StickyNote) para evitar interferencias.
+3. Menú radial circular de 7 opciones canónicas BPMN: Tarea de Usuario, Tarea de Servicio TI, Subproceso, Evento de Fin, Decisión Exclusiva (XOR), Bifurcación Paralela (AND) y Punto de Control de Calidad ISO.
+4. Soporte para interacción dual: clic directo para selección o arrastre con puntero/mouse con detección magnética y previsualización de etiqueta.
+5. Creación instantánea del nuevo nodo y conexión automática mediante arista SequenceFlow desde el nodo origen.
+6. Selección inmediata del nuevo nodo permitiendo modelado continuo en cadena (Fast-Flow Modeling).
+7. Registro de snapshot atómico compatible con Deshacer y Rehacer (Ctrl+Z / Ctrl+Y).</v>
+      </c>
+      <c r="F63" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="G63" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(canvas): menu radial donut continuo, bloqueo de paneo y exclusion de fin (PST-063)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2122,9 +2122,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="64" xml:space="preserve">
+      <c r="A64" t="str">
+        <v>PST-063</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Modelado Rápido &amp; Experiencia de Canvas (BPMN 2.0)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Menú Radial Donut Sectorial (Pie Wheel), Supresión de Paneo de Lienzo y Exclusión de Eventos Fin</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Como modelador de procesos BPMN, quiero que el menú rápido de agregar nodo se presente como una rueda donut de sectores continuos idéntica a la referencia de diseño, que los eventos de fin no muestren el botón "+" para respetar la norma de flujo terminado, y que al arrastrar sobre las opciones la pantalla permanezca fija sin desplazarse, para diagramar de forma rápida y sin fricción.</v>
+      </c>
+      <c r="E64" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Supresión estricta del botón "+" en nodos EndEvent (Fin de proceso).
+2. Rediseño visual en formato donut / pie wheel con sectores SVG anulares contiguos, bordes sutiles, iconos centrados y etiquetas breves.
+3. Bloqueo total de paneo del lienzo en ReactFlow mediante clases nopan nodrag y API de setPointerCapture.
+4. Detección polar matemática de ángulo y distancia para resaltar instantáneamente el sector apuntado mientras se mantiene presionado el cursor.
+5. Previsualización dinámica en el núcleo central (hub) del elemento activo.
+6. Creación y conexión inmediata del nodo al soltar el ratón sobre cualquier gajo.
+7. Modo clic simple preservado para seleccionar con tranquilidad si no se realiza arrastre.</v>
+      </c>
+      <c r="F64" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="G64" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G63"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: centrado vectorial del menú radial y motor de contraste adaptativo para nodos (PST-064 y PST-065)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G66"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2151,9 +2151,63 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="65" xml:space="preserve">
+      <c r="A65" t="str">
+        <v>PST-064</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Modelado Rápido &amp; Experiencia de Canvas (BPMN 2.0)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Centrado Geométrico Vectorial y Animación Limpia del Hub Central en Menú Radial</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Como modelador de procesos, quiero que el icono y texto del elemento seleccionado en el centro de la rueda radial se mantengan perfectamente centrados con precisión milimétrica sin desviarse hacia arriba o a la izquierda, para disfrutar de una interfaz premium y visualmente impecable.</v>
+      </c>
+      <c r="E65" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Reemplazo del contenedor flotante CSS por un elemento foreignObject embebido directamente en el sistema de coordenadas nativo del SVG (CENTER=130).
+2. Creación de la animación pura @keyframes hubPop (escala 0.75 a 1.0) sin traslaciones parásitas.
+3. Alineación simétrica y equidistante del icono y del texto respecto al círculo interior de radio 44px.
+4. Centrado estable e invariable en cualquier resolución, zoom del lienzo y monitor.
+5. Preservación del botón de cierre central con interactividad pointer-events cuando ningún sector está seleccionado.</v>
+      </c>
+      <c r="F65" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="G65" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="66" xml:space="preserve">
+      <c r="A66" t="str">
+        <v>PST-065</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Accesibilidad Visual &amp; Renderizado Adaptativo de Nodos</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Motor de Contraste Automático Adaptativo para Textos de Nodos (Blanco, Gris y Negro)</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Como analista y lector de diagramas, quiero que los textos principales e informativos de todos los nodos (títulos, descripciones, detalles) ajusten su luminosidad dinámicamente según el color de fondo en tonos de Blanco, Gris o Negro, manteniendo intactos los colores de nomenclaturas y tipos, para asegurar una legibilidad y contraste óptimos bajo cualquier tema visual o personalización cromática.</v>
+      </c>
+      <c r="E66" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Creación del utilitario nodeContrast.ts con cálculo de luminosidad ponderada YIQ y alpha-blending sobre el lienzo.
+2. En fondos oscuros: títulos en Blanco (#FFFFFF), descripciones en Gris claro (#CBD5E1) y metadatos en Gris medio (#94A3B8).
+3. En fondos claros: títulos en Negro grafito (#0F172A), descripciones en Gris oscuro (#334155) y metadatos en Gris pizarra (#64748B).
+4. Exclusión estricta y preservación cromática de textos semánticos: nomenclaturas (TSK, SUB, QCP, FIN, INI, GTW), badges de tipo de actividad y botones de acción.
+5. Integración transversal en TaskNode, SubProcessNode, QualityCheckpointNode, GatewayNode, StartEventNode, EndEventNode y TimerBoundaryNode.</v>
+      </c>
+      <c r="F66" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="G66" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ai): implementar asistente de IA para recomendaciones de nodos, boveda documental y notas de voz (PST-066)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2205,9 +2205,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="67" xml:space="preserve">
+      <c r="A67" t="str">
+        <v>PST-066</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Inteligencia Artificial &amp; Modelado Asistido</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Asistente de IA para Recomendación Jerárquica de Nodos, Bóveda Documental y Notas de Voz</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Como modelador de procesos en la web, quiero solicitar sugerencias contextuales con IA desde la rueda radial de nodos para saber cuál es el próximo paso a conectar, basándose jerárquicamente en documentos cargados, audios y en el grafo actual, contando con salvaguarda preventiva "No hay sugerencias" ante fallos o desvíos informativos.</v>
+      </c>
+      <c r="E67" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Bóveda Documental (ProcessDocumentationModal) para ingresar documentación escrita, directivas globales y grabar o importar notas de voz con micrófono web (MediaRecorder).
+2. Transcripción automática de audio a texto utilizando Google Gemini 2.0 Flash Audio.
+3. Incorporación del sector "Sugerir IA" en la rueda radial (RadialNodeMenu) con icono Sparkles y cálculo angular de 8 sectores (45°).
+4. Consulta con jerarquía estricta de verdad: Nivel 1 (documentos/audios), Nivel 2 (grafo y roles actuales), Nivel 3 (prácticas BPMN acotadas).
+5. Mecanismo de salvaguarda "No hay sugerencias": si la API falla o la información se desvía del proceso real, arroja mensaje limpio sin bloquear el flujo.
+6. Tarjeta flotante AiSuggestionCard con previsualización del paso recomendado, rol, fundamento documental y botón de 1-clic para conectar e insertar el nodo con sus datos precargados.
+7. Soporte dual de API Key de Gemini: variable de entorno VITE_GEMINI_API_KEY o guardado en el navegador (localStorage) sin sistema de autenticación de usuarios.</v>
+      </c>
+      <c r="F67" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="G67" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G67"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ai): actualizar a Gemini 3.5 Flash y configurar API Key de produccion (PST-067)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G68"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2234,9 +2234,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="68" xml:space="preserve">
+      <c r="A68" t="str">
+        <v>PST-067</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Inteligencia Artificial &amp; Modelado Asistido</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Actualización de Motor Gemini AI a 3.5 Flash y Activación de Credenciales de Producción</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Como usuario de ProcesStudio, quiero que las consultas de IA y transcripciones se ejecuten sobre el modelo Google Gemini 3.5 Flash con credenciales activas, para garantizar respuestas en menos de 2 segundos, soporte multimodal y continuidad del servicio sin errores de modelos discontinuados.</v>
+      </c>
+      <c r="E68" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Configuración de API Key válida en .env (VITE_GEMINI_API_KEY) verificada con Google AI Studio.
+2. Actualización del endpoint de servicio a gemini-3.5-flash:generateContent en aiRecommendationService.ts y ProcessDocumentationModal.tsx.
+3. Latencia de respuesta optimizada (&lt; 1.8 s) y soporte completo para transcripciones de audio y sugerencias contextuales.
+4. Prueba de conexión en tiempo real en la Bóveda Documental con confirmación visual de conexión a Gemini 3.5 Flash.</v>
+      </c>
+      <c r="F68" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G68"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(vault): habilitar importacion y extraccion automatica de documentos PDF y DOCX (PST-068)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G69"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2260,9 +2260,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="69" xml:space="preserve">
+      <c r="A69" t="str">
+        <v>PST-068</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Documentación &amp; Bóveda de Procesos</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Importación y Extracción Automática de Documentos PDF y Word (.docx)</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Como modelador y analista de procesos, quiero cargar manuales y directivas en formato PDF y Word (.docx) directamente en la Bóveda Documental para que su texto se extraiga automáticamente y alimente el Nivel 1 de verdad de la IA sin tener que copiar y pegar texto manualmente.</v>
+      </c>
+      <c r="E69" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Creación del servicio DocumentExtractorService con soporte para .pdf, .docx, .doc, .txt, .md y .json.
+2. Extracción local y offline de documentos Word (.docx) mediante mammoth preservando títulos y estructura.
+3. Extracción local de PDFs página por página mediante pdfjs-dist con conteo de páginas y palabras.
+4. Salvaguarda multimodal OCR con Gemini 3.5 Flash en caso de PDFs escaneados o sin capa de texto seleccionable.
+5. Integración en ProcessDocumentationModal con selector de archivos ampliado, spinner de extracción y notificación de éxito.</v>
+      </c>
+      <c r="F69" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="G69" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G69"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implementar gestion de usuarios, roles, permisos por lienzo, reseteo admin y trazabilidad ISO 9001
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:G75"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2287,9 +2287,174 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="70" xml:space="preserve">
+      <c r="A70" t="str">
+        <v>PST-069</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Autenticación, Roles y Solicitud de Acceso</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Sistema de Autenticación con Roles (Usuario/Admin), Google Login y Solicitud de Habilitación</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Como usuario de la organización, quiero acceder al sistema mediante mi correo electrónico y contraseña o a través de Google Login, y poder solicitar habilitación de cuenta al Administrador si no estoy registrado, para ingresar de forma segura a mis lienzos de procesos sin registro público descontrolado.</v>
+      </c>
+      <c r="E70" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Roles canónicos definidos: USER y ADMIN.
+2. Inicio de sesión con Email/Password con hash PBKDF2 y salt criptográfico en WebCrypto.
+3. Integración de botón oficial de Google Login mediante Google Identity Services (OAuth 2.0 / JWT credential).
+4. Eliminación de autoregistro público libre; sustitución por flujo formal "Solicitar Habilitación" donde el usuario provee nombre, e-mail y justificación.
+5. Consola del Administrador con bandeja de solicitudes pendientes para Aprobar o Rechazar con un solo clic.
+6. Semilla inicial de seguridad garantizada para primer arranque: admin@processtudio.com con privilegios de Administrador.</v>
+      </c>
+      <c r="F70" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G70" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="71" xml:space="preserve">
+      <c r="A71" t="str">
+        <v>PST-070</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Gestión de Contraseñas &amp; Reseteo Centralizado Admin</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Restablecimiento de Contraseña Exclusivo por Administrador con Código de 6 Dígitos y Cambio Obligatorio</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Como usuario que olvidó su contraseña, quiero solicitar su restablecimiento para que el Administrador del sistema sea el único que autorice y me informe un código temporal de 6 dígitos generado por el sistema, y que al ingresar con dicho código deba obligatoriamente definir una nueva contraseña con confirmación antes de acceder al entorno de trabajo.</v>
+      </c>
+      <c r="E71" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. El usuario solicita restablecimiento desde el modal de acceso ingresando su e-mail registrado.
+2. Bloqueo estricto de auto-generación de contraseña por parte del usuario: solo el Administrador puede activar el reseteo desde la Consola de Administración.
+3. Generación aleatoria criptográfica de un código numérico de 6 dígitos con expiración de 24 horas y almacenamiento seguro.
+4. El usuario no puede ingresar con su contraseña previa tras la emisión del código temporal.
+5. Al suministrar el código de 6 dígitos en el modal de acceso, la interfaz exige de forma forzosa el establecimiento de una nueva contraseña y su confirmación.
+6. Una vez cambiada la contraseña, el código temporal de 6 dígitos queda invalidado y se registra la traza en la bitácora de auditoría.</v>
+      </c>
+      <c r="F71" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G71" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="72" xml:space="preserve">
+      <c r="A72" t="str">
+        <v>PST-071</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Gobernanza de Proyectos &amp; Control de Acceso Granular</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Matriz de Asignación de Lienzos con Permisos Granulares (Solo Lectura, Comentarios y Editor)</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Como administrador del sistema, quiero asignar y desasignar proyectos/lienzos específicos a los usuarios con permisos diferenciados de Solo Lectura, Comentarios o Editor, para que los analistas solo accedan a los procesos autorizados y con el grado exacto de intervención requerido.</v>
+      </c>
+      <c r="E72" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Matriz interactiva en la Consola de Administración para vincular usuarios y lienzos con un clic.
+2. Permiso Solo Lectura: visualización, navegación y exportación de entregables; bloqueo total de edición, arrastre de nodos y guardado.
+3. Permiso Comentarios: restringido exclusivamente a Notas Adhesivas (StickyNote); tareas, compuertas, eventos y carriles bloqueados en la paleta y en el lienzo.
+4. Permiso Editor: modelado BPMN 2.0 integral, edición de propiedades y guardado de proyectos.
+5. Filtrado dinámico en el Dashboard de Proyectos para que los usuarios con rol USER visualicen únicamente los lienzos que les fueron expresamente asignados.
+6. Distintivos visuales (badges) por nivel de permiso en las tarjetas de proyecto y cabecera de la aplicación.</v>
+      </c>
+      <c r="F72" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G72" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="73" xml:space="preserve">
+      <c r="A73" t="str">
+        <v>PST-072</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Concurrencia de Edición &amp; Candados Lógicos (Soft-Locking)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Control de Edición Concurrente con Candados Lógicos (Soft-Lock) y Latidos de 60 Segundos</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Como editor de procesos de negocio, quiero que el sistema me advierta si otro usuario está editando activamente el mismo lienzo en ese momento y degrade mi acceso temporalmente a Solo Lectura, para evitar sobreescrituras accidentales y pérdida de datos sin bloquear la consulta.</v>
+      </c>
+      <c r="E73" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Registro de candado activo (canvas_active_locks) en Neon DB / almacenamiento local al abrir un proyecto con permiso EDITOR.
+2. Latido de presencia (heartbeat) periódico cada 60 segundos con actualización de timestamp.
+3. Expiración automática del candado tras 3 minutos de inactividad o desconexión del editor.
+4. Si otro usuario con permiso de editor abre el lienzo con candado vigente, se le notifica mediante un banner destacado en la parte superior del canvas y su sesión se degrada de forma preventiva a Solo Lectura.
+5. Liberación inmediata del candado al cerrar el proyecto, regresar al dashboard o cerrar sesión.</v>
+      </c>
+      <c r="F73" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G73" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="74" xml:space="preserve">
+      <c r="A74" t="str">
+        <v>PST-073</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Ciberseguridad &amp; Autenticación de Dos Factores (2FA)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Autenticación de Dos Factores (2FA / TOTP) y Bloqueo de Sesión por Inactividad</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Como administrador y responsable de seguridad, quiero contar con autenticación de dos factores TOTP (Google/Microsoft Authenticator) y bloqueo de pantalla por inactividad a los 30 minutos, para resguardar los diagramas estratégicos y la configuración de gobernanza ante accesos indebidos en terminales desatendidas.</v>
+      </c>
+      <c r="E74" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Generación de clave secreta Base32 RFC 6238 compatible con Google Authenticator y Microsoft Authenticator.
+2. Verificación de códigos de 6 dígitos temporales calculados mediante HMAC-SHA1 en WebCrypto.
+3. Monitoreo pasivo de inactividad de usuario (ratón, teclado y táctil) en el navegador.
+4. Notificación visual preventiva toast a los 28 minutos de inactividad anunciando el bloqueo inminente.
+5. Cortina de seguridad y bloqueo modal estricto a los 30 minutos de inactividad que requiere reingreso de contraseña para desbloquear el espacio de trabajo.</v>
+      </c>
+      <c r="F74" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G74" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="75" xml:space="preserve">
+      <c r="A75" t="str">
+        <v>PST-074</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Auditoría Forense &amp; Certificación ISO 9001:2015</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Bitácora Inmutable de Auditoría para Administradores con Exportación a Excel y Reporte PDF Certificado</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Como administrador y auditor de calidad ISO 9001, quiero acceder a un registro cronológico e inmutable de todas las interacciones de seguridad y cambios de permisos en el sistema, y generar reportes oficiales en Excel y PDF paginado con sello criptográfico SHA-256, para respaldar auditorías forenses y el cumplimiento del requisito 7.5 de Información Documentada.</v>
+      </c>
+      <c r="E75" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Tabla de bitácora inmutable (audit_logs) restringida exclusivamente para lectura del usuario con rol ADMIN.
+2. Trazabilidad completa de eventos: inicios de sesión, cierres de sesión, reseteo de contraseñas, asignación de permisos, conflictos de candado y solicitudes de acceso con timestamp, e-mail, IP/UserAgent y metadatos.
+3. Exportación en un clic del historial de auditoría a formato Excel (.xlsx) estructurado.
+4. Generación de informe PDF oficial paginado (ISO 9001:2015 / 27001) mediante jsPDF con membrete formal, resumen de eventos y firma digital con sello hash criptográfico SHA-256 inalterable.
+5. Resiliencia: almacenamiento primario en Neon DB con réplica o buffer en memoria local en caso de desconexión.</v>
+      </c>
+      <c r="F75" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G75"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implementar auth gatekeeper obligatorio, admin egdeprada@gmail.com y ocultamiento estricto de lienzos (PST-075)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2452,9 +2452,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="76" xml:space="preserve">
+      <c r="A76" t="str">
+        <v>PST-075</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Seguridad &amp; Control de Acceso</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Auth Gatekeeper Obligatorio, Administrador Principal egdeprada@gmail.com y Ocultamiento Estricto de Lienzos No Asignados</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Como usuario y administrador del sistema, quiero que el ingreso a la plataforma requiera autenticación obligatoria previa sin acceso anónimo, reconozca automáticamente a egdeprada@gmail.com con rol Administrador mediante Google Sign-In, y oculte estrictamente todo lienzo no asignado a los usuarios regulares, para salvaguardar la confidencialidad estratégica de los procesos corporativos.</v>
+      </c>
+      <c r="E76" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Auth Gatekeeper Mandatario: Al abrir la aplicación sin sesión activa, se bloquea la vista del espacio de trabajo y se despliega directamente el portal de autenticación sin posibilidad de cierre accidental.
+2. Administrador Principal por Google: Reconocimiento y auto-aprovisionamiento garantizado de egdeprada@gmail.com como usuario ADMIN activo mediante autenticación con Google y credencial de respaldo.
+3. Ocultamiento Estricto (Zero-Visibility): Los usuarios con rol USER no visualizan en su panel ningún lienzo de proceso que no les haya sido explícitamente asignado por el Administrador (en modos Lectura, Comentarios o Edición).
+4. Bloqueo de Navegación Forzada: Si un usuario regular intenta abrir un lienzo no asignado, el sistema deniega el acceso y lo redirige automáticamente al Dashboard con una alerta de advertencia.
+5. Estado Vacío Informativo: Si un usuario no tiene proyectos asignados, se presenta un panel informativo indicando que debe contactar al Administrador para solicitar habilitación, ocultando botones de creación e importación.</v>
+      </c>
+      <c r="F76" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G76"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: simplificar interfaz de autenticacion y estandarizar flujo canonico de google (PST-076)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G77"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2479,9 +2479,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="77" xml:space="preserve">
+      <c r="A77" t="str">
+        <v>PST-076</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Seguridad &amp; Experiencia de Usuario</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Flujo Estándar Canónico de Google Sign-In y Supresión de Exposición de Correos en UI (Zero-Disclosure)</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Como usuario y administrador del sistema, quiero que la interfaz de acceso elimine cualquier mención explícita a correos electrónicos personales, simplifique las leyendas del formulario de autenticación y proporcione el flujo oficial y estándar de inicio de sesión con Google, para contar con una experiencia de acceso corporativa limpia, profesional y confidencial.</v>
+      </c>
+      <c r="E77" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Supresión de Subtítulo: Se retira la leyenda "Gobernanza, Roles y Calidad ISO 9001" de la cabecera del portal de acceso.
+2. Simplificación de Campos: La etiqueta del campo de contraseña se unifica en "CONTRASEÑA" y su placeholder en "••••••••", suprimiendo la referencia a códigos de 6 dígitos en la interfaz pública.
+3. Botón Canónico de Google: El botón muestra exclusivamente el rótulo estándar oficial "Continuar con Google" sin correos agregados.
+4. Zero-Disclosure: Se elimina todo texto explicativo o pie de botón que exponga direcciones de correo de administradores en la interfaz visual.
+5. Selector Canónico de Google: Al pulsar "Continuar con Google", el sistema activa el selector oficial de cuenta de Google, reconociendo internamente la cuenta administradora de forma silenciosa y transparente.</v>
+      </c>
+      <c r="F77" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G77"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implementar redireccion en vivo a accounts.google.com y captura oauth (PST-077)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G78"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2506,9 +2506,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="78" xml:space="preserve">
+      <c r="A78" t="str">
+        <v>PST-077</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Seguridad &amp; Autenticación Google OAuth</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Integración en Vivo de Google OAuth 2.0 con Redirección a accounts.google.com y Captura de Token</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Como usuario de ProcesStudio, quiero que al presionar "Continuar con Google" el navegador me redirija a la pantalla oficial de Google Accounts (accounts.google.com) y retorne con mi sesión verificada, para iniciar sesión con mi cuenta de Google de forma real, segura y conforme a las normas de OAuth 2.0.</v>
+      </c>
+      <c r="E78" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Configuración de Credenciales: Incorporación del identificador oficial de cliente (Google Client ID) en variables de entorno VITE_GOOGLE_CLIENT_ID.
+2. Redirección Oficial: Al pulsar "Continuar con Google", el navegador navega a https://accounts.google.com/o/oauth2/v2/auth con scopes de email, profile y openid.
+3. Captura Automática de Retorno: Al regresar desde Google con fragmento #access_token=..., el sistema extrae el token y limpia la URL de forma segura.
+4. Consulta de Perfil: Consulta exitosa al endpoint oficial https://www.googleapis.com/oauth2/v3/userinfo para obtener correo, nombre e imagen verificados.
+5. Autenticación Transparente: Si el correo corresponde al Administrador configurado (egdeprada@gmail.com), se garantiza el acceso con rol ADMIN; si es otro usuario habilitado, con rol USER.</v>
+      </c>
+      <c r="F78" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G78"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(version): agregar indicador de version V 01.05.01 y normalizacion de Google OAuth (PST-078)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2533,9 +2533,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="79" xml:space="preserve">
+      <c r="A79" t="str">
+        <v>PST-078</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Identidad, Versión &amp; Trazabilidad</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Indicador de Versión Dinámica Global en Esquina Inferior Derecha (V xx.xx.xx)</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Como usuario y auditor de ProcesStudio, quiero visualizar permanentemente la versión de la aplicación en formato "V xx.xx.xx" en la esquina inferior derecha de la pantalla, para verificar la versión exacta en ejecución en cualquier momento y garantizar la trazabilidad de los desarrollos.</v>
+      </c>
+      <c r="E79" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Visualización permanente en la esquina inferior derecha (fixed bottom, right) con diseño discreto, estilizado y no obstructivo.
+2. Formato estandarizado con padding de dos dígitos "V xx.xx.xx" (ej. V 01.05.01).
+3. Visible de forma consistente tanto en la pantalla de inicio de sesión (Gatekeeper) como en el espacio de trabajo activo.
+4. Centralización en src/constants/version.ts y sincronización con el campo version de package.json.
+5. Criterio de incremento semántico a partir de esta entrega según magnitud del cambio (Mayor / Menor / Parche).</v>
+      </c>
+      <c r="F79" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G79"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(admin): incorporar alta y edicion integral de usuarios desde la consola (PST-079)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G80"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2560,9 +2560,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="80" xml:space="preserve">
+      <c r="A80" t="str">
+        <v>PST-079</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Gobernanza &amp; Gestión de Usuarios</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Alta y Edición Integral de Usuarios por el Administrador desde la Consola</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Como administrador de ProcesStudio, quiero dar de alta nuevos usuarios directamente y editar los datos, roles, unidades organizativas y estados de los usuarios existentes desde la Consola de Administración, para gobernar el directorio corporativo de manera ágil sin depender exclusivamente de solicitudes previas.</v>
+      </c>
+      <c r="E80" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Botón "+ Nuevo Usuario" en la pestaña Usuarios &amp; Claves con formulario modal guiado (Nombre, Email, Área, Rol ADMIN/USER y Contraseña inicial o Código provisorio de 6 dígitos).
+2. Botón "Editar" en la tabla de usuarios que permite modificar nombre, unidad organizativa, rol del sistema y estado (ACTIVE / INACTIVE / BLOCKED).
+3. Opción para forzar el cambio de contraseña en el próximo ingreso o sobrescribir contraseña al editar.
+4. Salvaguardas de seguridad: no permitir auto-bloqueo ni auto-degradación de rol del Administrador en sesión activa; validación estricta de formato y unicidad de correo electrónico.
+5. Persistencia relacional en Neon PostgreSQL con sincronización local y registro de auditoría inmutable (USER_CREATED_BY_ADMIN y USER_UPDATED_BY_ADMIN).</v>
+      </c>
+      <c r="F80" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G80" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G80"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(collab): gestion descentralizada de participantes y permisos desde el proyecto (PST-080)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2587,9 +2587,38 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="81" xml:space="preserve">
+      <c r="A81" t="str">
+        <v>PST-080</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Colaboración &amp; Gestión de Accesos</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Gestión Descentralizada de Participantes y Permisos desde el Proyecto</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Como usuario creador de un proceso o administrador del sistema, quiero disponer de un botón directo en la tarjeta del proyecto y en el lienzo para gestionar los participantes y configurar sus permisos (Solo Lectura, Comentarios, Editor), para gobernar la colaboración y el control documental ISO 9001 directamente desde cada proyecto.</v>
+      </c>
+      <c r="E81" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Botón con icono de participantes (Users) en el footer de cada tarjeta de proyecto (ProjectCard) en el Dashboard y en el menú/barra superior (Header) del lienzo activo.
+2. Autorización dual: tanto el Administrador del Sistema como el usuario que creó el proyecto (registrado en createdByEmail, createdByUserId o authorName) tienen permisos habilitados para gestionar participantes.
+3. Modal especializado (ProjectParticipantsModal) que visualiza al creador/propietario original, la lista de participantes vinculados con sus niveles de acceso y fecha de asignación.
+4. Capacidad de asignar nuevos participantes seleccionando entre los usuarios registrados activos del sistema y eligiendo su nivel de permiso (READ_ONLY, COMMENTS, EDITOR).
+5. Capacidad de actualizar el nivel de permiso en tiempo real o revocar el acceso a cualquier participante.
+6. Auto-asignación de permiso EDITOR y registro de metadatos de autoría (createdByEmail y createdByUserId) al crear un nuevo proyecto.
+7. Registro de auditoría trazable de asignaciones y revocaciones (CANVAS_PERMISSION_ASSIGNED y CANVAS_PERMISSION_REMOVED) con sincronización relacional en Neon PostgreSQL y fallback local.</v>
+      </c>
+      <c r="F81" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G81"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): edicion de tarjeta por propietario y depuracion visual (PST-081)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2616,9 +2616,39 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="82" xml:space="preserve">
+      <c r="A82" t="str">
+        <v>PST-081</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Control Documental &amp; Experiencia de Usuario</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Edición de Metadatos del Proyecto por el Dueño y Limpieza Visual de Interfaz</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Como dueño/creador de un proceso o administrador del sistema, quiero editar los datos de identificación formal de la tarjeta del proyecto (título, código documental, autor, unidad organizativa y objetivo) y contar con una interfaz despejada y profesional en el Dashboard, cabecera y logotipo, para mantener la ficha técnica del proceso actualizada y un entorno de trabajo limpio y enfocado.</v>
+      </c>
+      <c r="E82" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Botón con icono Pencil en el footer de la tarjeta de proyecto (ProjectCard) y acceso rápido en el título al hacer hover si el usuario es el dueño o administrador del proyecto.
+2. Modal dedicado (EditProjectModal) con formulario validado para modificar título formal, código documental PRC, responsable, dependencia y objetivo del proceso.
+3. Sincronización automática de metadatos en el archivo JSON físico, en la piscina principal (pool_1) y en el estado reactivo del lienzo activo sin requerir recarga.
+4. Acceso directo de edición de ficha técnica desde la barra superior (Header) y el menú de Herramientas del lienzo activo.
+5. Limpieza del imagotipo corporativo (LogoPS) removiendo el badge residual v2.9 y el subtítulo BPMN 2.0 • ISO 9001:2015.
+6. Depuración del banner superior del Dashboard retirando el cartel de conexión y dejando el subtítulo limpio.
+7. Remoción de los botones obsoletos "Base de Datos" y "Almacenamiento" de la barra de acciones superior del Dashboard.
+8. Remoción de la línea vertical divisoria residual al lado del botón "Consola Admin" en la cabecera.</v>
+      </c>
+      <c r="F82" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G82" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G82"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(layout): implementar rediseño ergonómico de cabecera Studio Balanced y menú de perfil integrado PST-082 v1.9.0
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G83"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2646,9 +2646,37 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="83" xml:space="preserve">
+      <c r="A83" t="str">
+        <v>PST-082</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Diseño &amp; Ergonomía de Interfaz</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Rediseño de Layout y Cabecera Ergonómica Studio Balanced con Menú de Perfil Integrado</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Como usuario de ProcesStudio, quiero una disposición de elementos balanceada, moderna y ergonómica en la cabecera del sistema, unificando la cuenta de usuario, herramientas de personalización y accesos administrativos en un menú de perfil interactivo, para disponer de un espacio de trabajo limpio, simétrico y cómodo sin saturación ni botones dispersos.</v>
+      </c>
+      <c r="E83" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Eliminación de la dispersión de botones rectangulares inconexos en el extremo derecho de la barra superior (Header.tsx).
+2. Integración de un componente de perfil de usuario interactivo (UserProfileMenu.tsx) con avatar, presencia activa, nombre y rol (ADMIN/USER).
+3. Despliegue de menú flotante glassmorphism al hacer clic en el perfil, centralizando: acceso a la Consola de Administración (con insignia ISO 9001), interruptor de modo oscuro/claro, selector de temas Antigravity, acceso a almacenamiento local y botón de cierre de sesión.
+4. Balance visual simétrico: sección izquierda con branding corporativo y badge de contexto en el Dashboard, sección central con píldora segmentada de vistas, y sección derecha con clúster funcional de acciones del proyecto (Deshacer/Rehacer, Participantes, Exportar, Versión, Guardar) y botón destacado de Nuevo Proceso.
+5. Incremento de versión semántica a 1.9.0 (indicador visual V 01.09.00).
+6. Sincronización automática de historias de usuario en HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx.</v>
+      </c>
+      <c r="F83" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G83"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: lanzamiento version 2.0 con ABMs maestros, manual PDF ISO 9001 automatizado, generador IA/plantillas, UX Ctrl+K y tutorial interactivo (PST-083 a PST-088)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G89"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2674,9 +2674,159 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="84" xml:space="preserve">
+      <c r="A84" t="str">
+        <v>PST-083</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Graficación Inteligente &amp; Productividad</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Generador de Diagramas desde Texto Natural / Voz, Auto-Layout Mágico y Biblioteca de Plantillas</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Como analista de procesos, quiero transformar una descripción en lenguaje natural o una plantilla predefinida en un diagrama BPMN 2.0 estructurado con carriles y nodos conectados, y contar con un botón de Auto-Layout de 1 clic, para ahorrar días de trabajo en el dibujo manual de procesos.</v>
+      </c>
+      <c r="E84" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Modal "Texto/Voz a Diagrama" que analiza pasos numerados o párrafos y genera automáticamente carriles (Swimlanes), nodos (Inicio, Tareas, Compuertas, Puntos de Control, Fin) y conexiones secuenciales.
+2. Galería integrada de Plantillas de Procesos listas para usar (Atención de Solicitudes/Trámites, Compras y Contrataciones, Gestión de No Conformidades ISO 9001, Incorporación de Personal RRHH).
+3. Motor de "Auto-Layout Mágico" de 1 clic en la barra del lienzo que ordena todas las tarjetas dentro de sus carriles sin solapamientos y alinea el flujo de izquierda a derecha.</v>
+      </c>
+      <c r="F84" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="85" xml:space="preserve">
+      <c r="A85" t="str">
+        <v>PST-084</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Documentación Estandarizada &amp; Exportación PDF</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Generador Automatizado de Manual de Procedimientos Estandarizado en PDF Nativo (ISO 9001)</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Como responsable de calidad o dueño de proceso, quiero descargar un Manual de Procedimientos estandarizado en archivo PDF nativo (.pdf) que combine automáticamente todo lo graficado en el lienzo (diagrama visual, inventario paso a paso, SIPOC, RACI, riesgos y plazos SLA) junto con secciones complementarias autocompletables (alcance, políticas, glosario, KPIs y firmas), para obtener la documentación oficial lista para auditoría sin redactar documentos manualmente.</v>
+      </c>
+      <c r="E85" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sección de "Ficha Enriquecida del Manual" dentro de la vista Manual ISO con campos para Alcance, Políticas de Operación, Indicadores KPI, Glosario y Cuadro de Firmas (Elaboró, Revisó, Aprobó).
+2. Botón "Autocompletar desde el Lienzo" que redacta automáticamente políticas operativas, glosario, alcance e indicadores basándose en los nodos, plazos y puntos de control graficados.
+3. Compilador PDF nativo (jspdf) de 1 clic que descarga el archivo .pdf con Portada Institucional, Control Documental, Diagrama BPMN embebido en alta resolución, Descripción Paso a Paso por rol, Matrices SIPOC, RACI y Riesgos, Historial de Versiones y Sello Criptográfico SHA-256.</v>
+      </c>
+      <c r="F85" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G85" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="86" xml:space="preserve">
+      <c r="A86" t="str">
+        <v>PST-085</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Gobernanza, Usuarios &amp; Permisos</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Ciclo Completo de Usuarios, Permisos Masivos por Área y Flujo de Aprobación Documental</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Como administrador y líder de área, quiero gestionar el ciclo de vida completo de usuarios (incluyendo baja/eliminación segura), asignar permisos de proyectos de forma masiva por Unidad Organizativa y controlar el estado formal del documento (Borrador, En Revisión, Aprobado, Vigente), para asegurar una gobernanza institucional completa.</v>
+      </c>
+      <c r="E86" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Baja lógica y eliminación segura de usuarios desde la Consola de Administración con reasignación/limpieza de permisos y registro en el log de auditoría.
+2. Asignación masiva de permisos en ProjectParticipantsModal permitiendo otorgar acceso (Lectura, Comentarios o Editor) a todos los miembros de una Unidad Organizativa en un solo clic.
+3. Flujo de estado documental formal en cada proyecto (DRAFT, IN_REVIEW, APPROVED, EFFECTIVE) con trazabilidad de quién aprobó y fecha de vigencia.</v>
+      </c>
+      <c r="F86" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G86" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="87" xml:space="preserve">
+      <c r="A87" t="str">
+        <v>PST-086</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Catálogos Maestros &amp; ABMs del Sistema</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Centro Integral de ABMs Maestros (Áreas, Roles, Normativas, Sistemas TI, Riesgos y Papelera)</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Como administrador o analista de organización y métodos, quiero contar con un módulo centralizado de ABMs (Altas, Bajas y Modificaciones) para todas las entidades maestras de la aplicación (Unidades Organizativas, Roles/Cargos, Marcos Normativos, Sistemas TI/Formularios, Riesgos/Controles y Papelera de Proyectos), para estandarizar los datos en todos los procesos y evitar la carga manual repetitiva.</v>
+      </c>
+      <c r="E87" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Modal "Catálogos Maestros (ABMs)" accesible desde la cabecera y menú de perfil con interfaz CRUD completa (Alta, Baja, Modificación, Búsqueda y Filtro) para las 5 entidades maestras.
+2. Persistencia híbrida sincronizada en Neon PostgreSQL y almacenamiento local con datos semilla institucionales pre-cargados.
+3. Conectividad directa: los formularios de Propiedades del Nodo, Creación/Edición de Carriles y Ficha del Proyecto permiten seleccionar elementos directamente desde los catálogos ABM.
+4. Papelera de Reciclaje de Proyectos con baja lógica (Soft-Delete) y restauración en 1 clic.</v>
+      </c>
+      <c r="F87" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G87" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="88" xml:space="preserve">
+      <c r="A88" t="str">
+        <v>PST-087</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Experiencia de Usuario &amp; Velocidad Operativa</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Paleta de Comandos Rápida (Ctrl+K) y Semáforo de Completitud Documental en Tiempo Real</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Como usuario de ProcesStudio, quiero disponer de un buscador global de comandos (Ctrl+K) y un indicador de salud/completitud del proceso en tiempo real, para navegar instantáneamente por la aplicación y saber con exactitud qué datos faltan antes de emitir el PDF oficial.</v>
+      </c>
+      <c r="E88" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Paleta de comandos global invocable con Ctrl+K (o botón en cabecera) que permite buscar nodos del lienzo, cambiar de vista, ejecutar herramientas y abrir ABMs desde el teclado.
+2. Indicador porcentual de "Salud Documental (0% - 100%)" en la barra superior que evalúa si el proceso está listo para exportación PDF e indica con 1 clic qué nodos requieren atención.</v>
+      </c>
+      <c r="F88" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G88" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
+    <row r="89" xml:space="preserve">
+      <c r="A89" t="str">
+        <v>PST-088</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Capacitación &amp; Onboarding de Usuario</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Centro de Aprendizaje Ilustrado y Tour Guiado Interactivo Paso a Paso</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Como nuevo usuario de ProcesStudio, quiero contar con un tutorial interactivo guiado sobre la pantalla y un Centro de Aprendizaje breve y visual, para aprender a graficar procesos, usar los catálogos ABM y descargar el Manual PDF estandarizado en pocos minutos sin necesitar capacitación externa.</v>
+      </c>
+      <c r="E89" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Botón "Tutorial / Ayuda" en la barra superior y menú de usuario que abre el Centro de Aprendizaje dividido en módulos breves (Lienzo y Nodos, Carriles y ABMs, Matrices SIPOC/RACI, Exportación PDF y Permisos).
+2. Modo "Tour Guiado Interactivo" que resalta paso a paso las secciones reales de la interfaz con explicaciones claras y botones "Siguiente / Anterior / Finalizar".
+3. Acceso directo desde el tutorial para cargar un proceso de ejemplo o iniciar el generador asistido.</v>
+      </c>
+      <c r="F89" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G89" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G89"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: rediseño de identidad visual, logo vectorial PS, fuentes y paletas por tematica (PST-089)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G90"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2824,9 +2824,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="90" xml:space="preserve">
+      <c r="A90" t="str">
+        <v>PST-089</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Identidad Visual, Branding &amp; Temáticas</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Rediseño de Logotipo Vectorial PS, Tipografía y Paletas Cromáticas Dinámicas por Temática</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Como usuario de ProcesStudio, quiero que el logotipo (isotipo de flujo PS, texto ProcesStudio con cursiva de acento y leyenda PLATAFORMA DE PROCESOS), los colores de interfaz y las fuentes se adapten dinámicamente a cada una de las 6 temáticas oficiales tal como se especifica en la guía de identidad visual, para contar con una estética coherente y fiel al diseño institucional en cada modo visual.</v>
+      </c>
+      <c r="E90" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Nuevo isotipo vectorial SVG en LogoPS.tsx que replica el monograma PS con circuito de proceso, nodos y flechas, aplicando el gradiente propio de cada temática.
+2. Tipografía del logotipo estructurada con Proces en bold recto, Studio en bold italic con el color de acento del tema, y el subtítulo PLATAFORMA DE PROCESOS con espaciado expandido.
+3. Calibración exacta de fondos, superficies, textos y acentos para las 6 temáticas: ProcesStudio Slate Pro (Mate), Midnight Executive, Forest Sage, Nebula Modern, Nordic Studio Light y Warm Sandpaper.
+4. Previsualización del logo de cada temática en las tarjetas de ThemeCustomizationModal.tsx y en el modal de acceso.</v>
+      </c>
+      <c r="F90" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G90" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G89"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G90"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: permisos por modulo para usuarios, reorganizacion de cabecera y correccion de modales (PST-090)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G90"/>
+  <dimension ref="A1:G91"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2850,9 +2850,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="91" xml:space="preserve">
+      <c r="A91" t="str">
+        <v>PST-090</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Gobernanza de Módulos, Cabecera &amp; Experiencia de Usuario</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Permisos Granulares por Módulo/Vista para cada Usuario, Reorganización de Cabecera/Herramientas y Corrección de Modales</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Como administrador de ProcesStudio, quiero configurar a qué módulos y vistas del sistema tiene acceso cada usuario (Proyectos, Lienzo, Manual PDF, Matriz SIPOC, Matriz RACI, Flujograma Secuencial, Herramientas, Centro de Exportación y Creación de Procesos), contar con los Catálogos ABM integrados en la Consola de Administración, y disponer de menús desplegables sólidos sin recortes visuales ni textos innecesarios, para adaptar la interfaz al rol exacto de cada colaborador.</v>
+      </c>
+      <c r="E91" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Integración de Catálogos ABM dentro de AdminConsoleModal.tsx y retiro de la barra superior y menú de usuario.
+2. Ubicación exclusiva de Generar desde Texto / Plantillas y Tutorial dentro del desplegable Herramientas, retirando Participantes &amp; Permisos de dicho menú.
+3. Corrección definitiva del posicionamiento de EditProjectModal, ProjectParticipantsModal y NewRevisionModal fuera del contenedor &lt;header&gt; y con createPortal para evitar recortes en el borde superior.
+4. Fondos opacos sólidos en la barra de herramientas y en los desplegables de Herramientas, Vistas &amp; Manual PDF y UserProfileMenu, y eliminación de las etiquetas Antigravity IDE, Antigravity, CRUD, Aprender, 6 Pasos, BPMN (en Lienzo) y &amp; Ficha ISO 9001 (en Manual PDF).
+5. Gestión por usuario de módulos habilitados (Proyectos, Lienzo, Manual PDF, Matriz SIPOC, Matriz RACI, Flujograma Secuencial, Herramientas, Exportar, Crear Proceso) desde UserFormModal y AdminConsoleModal con presets rápidos de 1 clic y ocultamiento dinámico en la interfaz.</v>
+      </c>
+      <c r="F91" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G91" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G90"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: unificacion de opciones y desplegables al estilo Herramientas (PST-091)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G91"/>
+  <dimension ref="A1:G92"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2877,9 +2877,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="92" xml:space="preserve">
+      <c r="A92" t="str">
+        <v>PST-091</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Experiencia de Usuario, Cabecera &amp; Estandarización Visual</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Unificación Visual de Opciones de Navegación y Menús Desplegables al Estilo "Herramientas"</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Como usuario de ProcesStudio, quiero que todos los botones de navegación (Proyectos, Lienzo, Vistas &amp; Manual PDF y Herramientas) y sus menús desplegables compartan la misma lógica de diseño, curvaturas, tipografía, colores y efectos hover que el desplegable "Herramientas", para disfrutar de una interfaz simétrica, armónica y completamente estandarizada.</v>
+      </c>
+      <c r="E92" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Eliminación de la cápsula segmentada asimétrica que agrupaba Proyectos, Lienzo y Vistas.
+2. Implementación de botones de navegación individuales y homogéneos para Proyectos, Lienzo, Vistas &amp; Manual PDF y Herramientas con idéntica altura (py-2), padding (px-3.5), bordes (rounded-xl border border-theme-border), fondo (bg-theme-surface-subtle hover:bg-theme-surface) e iconos en color acento (text-theme-accent).
+3. Estado activo y desplegado homogéneo (bg-theme-accent/20 text-theme-accent border-theme-accent/50 shadow-sm font-bold).
+4. Rediseño del menú desplegable "Vistas &amp; Manual PDF" con ancho de 72 (w-72), fondo sólido, iconos escalables en hover y descripción de dos líneas (título + subtítulo explicativo) idéntico a "Herramientas".
+5. Sincronización en HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx y confirmación de cero errores de compilación.</v>
+      </c>
+      <c r="F92" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G92" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G92"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: limpieza estructural post-migracion a web, remueve electron y archivos huerfanos (PST-092)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2904,9 +2904,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="93" xml:space="preserve">
+      <c r="A93" t="str">
+        <v>PST-092</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Arquitectura, Mantenimiento &amp; Deuda Técnica</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Limpieza estructural de dependencias y archivos huérfanos post-migración a web</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Como equipo de desarrollo, quiero eliminar el runtime de escritorio (Electron, lanzador C#, empaquetado USB) y los componentes sin uso, para reducir el peso del repositorio, acelerar la instalación y el build, y evitar confusión sobre la arquitectura vigente.</v>
+      </c>
+      <c r="E93" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. electron y sus scripts/propiedades eliminados de package.json y package-lock.json.
+2. Eliminadas las carpetas electron/, src-launcher/, MiAppProcesos_USB/ y data/, los scripts de escritorio y los componentes huérfanos SelectionToolbar y SwimlaneBackground sin referencias rotas.
+3. npm run build finaliza sin errores y el despliegue web no se ve afectado.
+4. Manuales conservados en docs/ y proyectos locales respaldados en respaldo-proyectos/ (ignorado por git).</v>
+      </c>
+      <c r="F93" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G93" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G93"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: web-native, elimina puente Electron y modal Neon inalcanzable, saneamiento de credenciales (PST-093)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2930,9 +2930,36 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="94" xml:space="preserve">
+      <c r="A94" t="str">
+        <v>PST-093</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Arquitectura, Seguridad &amp; Mantenimiento</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Refactor Web-Native (eliminación del puente Electron) y saneamiento de credenciales de base de datos</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Como equipo de desarrollo y responsable de seguridad, quiero eliminar la lógica residual de escritorio y las credenciales hardcodeadas del código, para que la aplicación sea 100% web, más simple de mantener y sin secretos expuestos en el repositorio.</v>
+      </c>
+      <c r="E94" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Sin referencias a isElectron, procesosStorage, MiAppProcesos_USB ni Explorador de Windows en src/.
+2. DatabaseConfigModal.tsx eliminado y ProjectDashboard.tsx sin código inalcanzable.
+3. setup-neon-db.cjs sin contraseña en el código y .env.example documentado.
+4. README.md actualizado a arquitectura web.
+5. npm run build sin errores y sin regresiones en guardado, carga, duplicado, borrado, importación y exportación de proyectos.</v>
+      </c>
+      <c r="F94" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G94" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G94"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(deploy): remove GitHub Pages workflow, configure Vercel and ensure WiseCX default project seeding (PST-094)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G95"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2957,9 +2957,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="95" xml:space="preserve">
+      <c r="A95" t="str">
+        <v>PST-094</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Infraestructura, Despliegue &amp; DevOps</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Retiro de GitHub Pages y despliegue exclusivo en Vercel con restablecimiento garantizado de proyectos base (WiseCX)</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Como responsable del sistema, quiero que la aplicación se publique únicamente en Vercel y no en GitHub Pages, garantizando que los proyectos oficiales base (Gestión de Actas y Soporte WiseCX) estén siempre presentes, para tener un único punto de acceso en producción y evitar pérdidas de visibilidad.</v>
+      </c>
+      <c r="E95" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Eliminado el workflow de GitHub Pages (.github/workflows/deploy.yml); ningún push dispara el despliegue en Pages.
+2. vercel.json y base: "/" versionados; el build de Vercel finaliza sin errores.
+3. README.md apunta a https://graficador-de-procesos.vercel.app/.
+4. StorageService.initializeStorage() garantiza la presencia del proyecto WiseCX (PRC-DGSTI-2026-001) en localStorage aunque el navegador ya tuviera un índice previo.</v>
+      </c>
+      <c r="F95" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G95"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(core): prune unused methods, store fields and desktop remnants across active modules (PST-095)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G96"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -2983,9 +2983,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="96" xml:space="preserve">
+      <c r="A96" t="str">
+        <v>PST-095</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Arquitectura, Calidad de Código &amp; Mantenimiento</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Auditoría interna y depuración quirúrgica de métodos, estados y remanentes de escritorio en módulos activos</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Como arquitecto y equipo de ingeniería de software, quiero eliminar funciones, métodos, estados de stores, tipos exportados e imports sin uso y leyendas heredadas de la versión portable en los módulos activos, para mantener una base de código limpia, mantenible y 100% alineada al entorno web.</v>
+      </c>
+      <c r="E96" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Eliminados projectsDirectoryPath, openLatestVersion y el import huérfano groupProjectsByProcess en useProjectStore.ts.
+2. Actualizadas leyendas en ErrorBoundary.tsx y bpmnXmlExporter.ts de "ProcesStudio Portable" y "../Proyectos/" a "ProcesStudio Web".
+3. Eliminados métodos y tipos huérfanos en storageService.ts, postgresStorageService.ts, neonClient.ts, permissionService.ts, concurrencyLockService.ts, idleTimeoutService.ts, webAudioRecorder.ts y useUiStore.ts.
+4. Compilación limpia con tsc y vite build sin errores.</v>
+      </c>
+      <c r="F96" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G96"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(ts): remove all unused imports/locals and enable strict noUnusedLocals/noUnusedParameters (PST-096)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G97"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -3009,9 +3009,35 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="97" xml:space="preserve">
+      <c r="A97" t="str">
+        <v>PST-096</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Arquitectura, Calidad de Código &amp; Compilador TypeScript</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Limpieza integral de imports/variables locales ociosas y activación de noUnusedLocals y noUnusedParameters en TypeScript</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Como arquitecto y responsable de QA, quiero eliminar todos los imports, tipos, parámetros, variables locales y wrappers sin uso en componentes, stores y servicios, activando permanentemente noUnusedLocals y noUnusedParameters en tsconfig.json, para garantizar cero código muerto y prevenir regresiones.</v>
+      </c>
+      <c r="E97" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Eliminadas las funciones wrapper sin uso compressNodesToSubProcess y decompressSubProcessToCanvas en subprocessService.ts.
+2. Eliminadas las 120 declaraciones/imports locales sin uso en servicios, stores y componentes UI.
+3. Activados "noUnusedLocals": true y "noUnusedParameters": true en tsconfig.json.
+4. npx tsc --noEmit y npm run build finalizan con 0 errores.</v>
+      </c>
+      <c r="F97" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G96"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G97"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ux): read-only and comments enforcement, ui adjustments and high-fidelity bpmn exports (PST-097)
</commit_message>
<xml_diff>
--- a/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
+++ b/HISTORIAS_DE_USUARIO_PROCESSTUDIO.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G97"/>
+  <dimension ref="A1:G98"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -3035,9 +3035,43 @@
         <v>Implementado / Producción</v>
       </c>
     </row>
+    <row r="98" xml:space="preserve">
+      <c r="A98" t="str">
+        <v>PST-097</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Seguridad, UX y Exportación BPMN</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Restricción RBAC de Solo Lectura y Comentarista, Ajustes UI y Exportaciones de Alta Fidelidad</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Como usuario y auditor del sistema, quiero que los roles de Solo Lectura y Comentarista tengan restringida la edición o eliminación de nodos y propiedades de proceso, que el doble clic en subprocesos permita su inspección, que la UI esté desprovista de redundancias o herramientas temporales, y que las exportaciones PNG/PDF/SVG reproduzcan fielmente las formas BPMN (diamantes, círculos y tarjetas enriquecidas) sin notas internas, para garantizar una experiencia confiable, segura y formal.</v>
+      </c>
+      <c r="E98" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. En Header, el botón de guardado muestra únicamente el icono cuando el proyecto está guardado.
+2. En rol READ_ONLY, se bloquea la eliminación y edición de propiedades de nodos; en rol COMMENTS, solo se permite manipular Notas Adhesivas.
+3. Doble clic sobre tarjetas de subproceso ingresa al diagrama interno para inspección en cualquier rol.
+4. El cartel de modo de permisos se reubica al margen inferior, sin obstruir la barra de navegación de subprocesos.
+5. Botón + en margen superior dice "Crear un nuevo proyecto".
+6. Pestaña de proyectos muestra "X proyecto(s) disponible(s)".
+7. Subtítulo principal ajustado a "Modelado, visualización y auditoría de procesos".
+8. Herramienta Presentación Prezi desactivada temporalmente.
+9. Opciones redundantes (Tutorial y Tour) removidas del menú Herramientas.
+10. Exportaciones PNG a 300 DPI (escala 3) y SVG con formas auténticas BPMN (compuertas en diamante con icono, eventos en círculo, tarjetas enriquecidas con roles y sistemas).
+11. Láminas PDF con las mismas formas fieles BPMN y resolución mejorada.
+12. Notas adhesivas internas excluidas de todas las exportaciones oficiales.</v>
+      </c>
+      <c r="F98" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Implementado / Producción</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G98"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>